<commit_message>
[fix] correction todo list
</commit_message>
<xml_diff>
--- a/todo.xlsx
+++ b/todo.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet state="visible" name="📋 TODO" sheetId="1" r:id="rId5"/>
-    <sheet state="visible" name="📊 RÉSUMÉ" sheetId="2" r:id="rId6"/>
-    <sheet state="visible" name="🔀 TABLEAU CROISÉ" sheetId="3" r:id="rId7"/>
+    <sheet state="visible" name=" TODO" sheetId="1" r:id="rId5"/>
+    <sheet state="visible" name=" RÉSUMÉ" sheetId="2" r:id="rId6"/>
+    <sheet state="visible" name="TABLEAU CROISÉ" sheetId="3" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr/>
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="353" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="323" uniqueCount="153">
   <si>
     <t>TACHE</t>
   </si>
@@ -48,6 +48,18 @@
     <t>INSCRIPTION</t>
   </si>
   <si>
+    <t>users.sql</t>
+  </si>
+  <si>
+    <t>Table users : id, nom, prenom, email, mdp, genre, taille, poids, imc, wallet, is_gold</t>
+  </si>
+  <si>
+    <t>SQL</t>
+  </si>
+  <si>
+    <t>Steeven</t>
+  </si>
+  <si>
     <t>register_step1.php</t>
   </si>
   <si>
@@ -57,81 +69,60 @@
     <t>HTML/CSS</t>
   </si>
   <si>
+    <t>Validation JS côté client : champs obligatoires, format email</t>
+  </si>
+  <si>
+    <t>JavaScript</t>
+  </si>
+  <si>
+    <t>register_step2.php</t>
+  </si>
+  <si>
+    <t>Design HTML/CSS formulaire étape 2 : taille (cm), poids (kg)</t>
+  </si>
+  <si>
+    <t>Calcul et affichage IMC en temps réel (AJAX)</t>
+  </si>
+  <si>
+    <t>JavaScript/AJAX</t>
+  </si>
+  <si>
+    <t>AuthController.php</t>
+  </si>
+  <si>
+    <t>Logique inscription 2 étapes : session entre pages, hash mdp, insertion BDD</t>
+  </si>
+  <si>
+    <t>PHP/CodeIgniter</t>
+  </si>
+  <si>
+    <t>LOGIN</t>
+  </si>
+  <si>
+    <t>login.php</t>
+  </si>
+  <si>
+    <t>Design page login : champs email + mot de passe + bouton</t>
+  </si>
+  <si>
+    <t>Mihaja</t>
+  </si>
+  <si>
+    <t>Logique login : vérif hash mdp, session CI4, logout, filtre auth</t>
+  </si>
+  <si>
+    <t>PROFIL</t>
+  </si>
+  <si>
+    <t>profile.php</t>
+  </si>
+  <si>
+    <t>Design page profil : affichage + formulaire édition</t>
+  </si>
+  <si>
     <t>Aina</t>
   </si>
   <si>
-    <t>Validation JS côté client : champs obligatoires, format email</t>
-  </si>
-  <si>
-    <t>JavaScript</t>
-  </si>
-  <si>
-    <t>register_step2.php</t>
-  </si>
-  <si>
-    <t>Design HTML/CSS formulaire étape 2 : taille (cm), poids (kg)</t>
-  </si>
-  <si>
-    <t>Mihaja</t>
-  </si>
-  <si>
-    <t>Calcul et affichage IMC en temps réel via AJAX</t>
-  </si>
-  <si>
-    <t>JavaScript/AJAX</t>
-  </si>
-  <si>
-    <t>AuthController.php</t>
-  </si>
-  <si>
-    <t>Logique inscription 2 étapes : stockage session entre pages</t>
-  </si>
-  <si>
-    <t>PHP/CodeIgniter</t>
-  </si>
-  <si>
-    <t>Steeven</t>
-  </si>
-  <si>
-    <t>Hash du mot de passe + insertion en base</t>
-  </si>
-  <si>
-    <t>users.sql</t>
-  </si>
-  <si>
-    <t>Table users : id, nom, prenom, email, mdp, genre, taille, poids, imc, wallet, is_gold</t>
-  </si>
-  <si>
-    <t>SQL</t>
-  </si>
-  <si>
-    <t>LOGIN</t>
-  </si>
-  <si>
-    <t>login.php</t>
-  </si>
-  <si>
-    <t>Design page login : champs email + mot de passe + bouton</t>
-  </si>
-  <si>
-    <t>Logique login : vérification hash mdp, création session CodeIgniter</t>
-  </si>
-  <si>
-    <t>Logique logout + destruction session</t>
-  </si>
-  <si>
-    <t>Middleware : redirection si non connecté (filter CI4)</t>
-  </si>
-  <si>
-    <t>PROFIL</t>
-  </si>
-  <si>
-    <t>profile.php</t>
-  </si>
-  <si>
-    <t>Design page profil : affichage infos + formulaire édition</t>
-  </si>
-  <si>
     <t>ProfileController.php</t>
   </si>
   <si>
@@ -153,7 +144,7 @@
     <t>ObjectifController.php</t>
   </si>
   <si>
-    <t>Sauvegarde objectif en session + base + redirection suggestion</t>
+    <t>Sauvegarde objectif en session + base + redirection vers suggestion</t>
   </si>
   <si>
     <t>SUGGESTION</t>
@@ -171,241 +162,244 @@
     <t>Algorithme sélection régimes selon IMC, objectif, delta_poids</t>
   </si>
   <si>
+    <t>Affichage prix avec/sans remise Gold (15%)</t>
+  </si>
+  <si>
+    <t>PHP/HTML</t>
+  </si>
+  <si>
+    <t>EXPORT PDF</t>
+  </si>
+  <si>
+    <t>export_pdf.php</t>
+  </si>
+  <si>
+    <t>Intégration bibliothèque TCPDF via Composer</t>
+  </si>
+  <si>
+    <t>PHP</t>
+  </si>
+  <si>
+    <t>Génération PDF : résumé régime + activités + IMC utilisateur</t>
+  </si>
+  <si>
+    <t>PORTE MONNAIE</t>
+  </si>
+  <si>
+    <t>wallet.php</t>
+  </si>
+  <si>
+    <t>Design page portefeuille : affichage solde + champ saisie code</t>
+  </si>
+  <si>
+    <t>WalletController.php</t>
+  </si>
+  <si>
+    <t>Vérification code AJAX : validation, crédit solde, marque utilisé</t>
+  </si>
+  <si>
+    <t>codes.sql</t>
+  </si>
+  <si>
+    <t>Table codes : id, code, montant, statut, user_id</t>
+  </si>
+  <si>
+    <t>OPTION GOLD</t>
+  </si>
+  <si>
+    <t>gold.php</t>
+  </si>
+  <si>
+    <t>Design page Gold : présentation avantages, prix, bouton achat</t>
+  </si>
+  <si>
+    <t>GoldController.php</t>
+  </si>
+  <si>
+    <t>Logique achat Gold : vérif solde, débit wallet, activation flag is_gold</t>
+  </si>
+  <si>
+    <t>Application automatique remise 15% si is_gold = 1</t>
+  </si>
+  <si>
+    <t>NAVIGATION</t>
+  </si>
+  <si>
+    <t>layout/navbar.php</t>
+  </si>
+  <si>
+    <t>Navbar front responsive : logo, liens, état connecté/déconnecté</t>
+  </si>
+  <si>
+    <t>layout/sidebar_bo.php</t>
+  </si>
+  <si>
+    <t>Sidebar back-office responsive avec liens vers toutes les sections</t>
+  </si>
+  <si>
+    <t>BO LOGIN</t>
+  </si>
+  <si>
+    <t>bo/login.php</t>
+  </si>
+  <si>
+    <t>Design + logique page authentification back-office, session admin</t>
+  </si>
+  <si>
+    <t>bo/AdminController.php</t>
+  </si>
+  <si>
+    <t>Middleware admin : vérif rôle, redirection si non autorisé</t>
+  </si>
+  <si>
+    <t>BO DASHBOARD</t>
+  </si>
+  <si>
+    <t>bo/dashboard.php</t>
+  </si>
+  <si>
+    <t>Design tableau de bord : cards KPI (nb users, CA, codes validés)</t>
+  </si>
+  <si>
+    <t>Graphe Chart.js : évolution inscriptions par mois (ligne)</t>
+  </si>
+  <si>
+    <t>Graphe Chart.js : répartition objectifs utilisateurs (camembert)</t>
+  </si>
+  <si>
+    <t>bo/DashboardController.php</t>
+  </si>
+  <si>
+    <t>Requêtes SQL pour KPI et données graphes (agrégats)</t>
+  </si>
+  <si>
+    <t>PHP/SQL</t>
+  </si>
+  <si>
+    <t>BO RÉGIMES</t>
+  </si>
+  <si>
+    <t>regimes.sql</t>
+  </si>
+  <si>
+    <t>Table régimes : id, nom, pct_viande, pct_poisson, pct_volaille, duree, prix, delta_poids</t>
+  </si>
+  <si>
+    <t>bo/regimes.php</t>
+  </si>
+  <si>
+    <t>Liste régimes : tableau paginé avec actions éditer/supprimer</t>
+  </si>
+  <si>
+    <t>bo/regimes_form.php</t>
+  </si>
+  <si>
+    <t>Formulaire création/édition : nom, % viande, % poisson, % volaille, durée, prix</t>
+  </si>
+  <si>
+    <t>bo/RegimeController.php</t>
+  </si>
+  <si>
+    <t>CRUD complet régimes avec validation (somme % = 100)</t>
+  </si>
+  <si>
+    <t>BO ACTIVITÉS</t>
+  </si>
+  <si>
+    <t>activites.sql</t>
+  </si>
+  <si>
+    <t>Table activités : id, nom, description, duree_min, calories_heure, niveau</t>
+  </si>
+  <si>
+    <t>bo/activites.php</t>
+  </si>
+  <si>
+    <t>Liste activités : tableau paginé avec actions éditer/supprimer</t>
+  </si>
+  <si>
+    <t>bo/activites_form.php</t>
+  </si>
+  <si>
+    <t>Formulaire création/édition activité sportive</t>
+  </si>
+  <si>
+    <t>bo/ActiviteController.php</t>
+  </si>
+  <si>
+    <t>CRUD complet activités sportives</t>
+  </si>
+  <si>
+    <t>BO CODES</t>
+  </si>
+  <si>
+    <t>bo/codes.php</t>
+  </si>
+  <si>
+    <t>Liste codes : tableau statut actif/utilisé + pagination</t>
+  </si>
+  <si>
+    <t>bo/codes_form.php</t>
+  </si>
+  <si>
+    <t>Formulaire génération de codes : montant, quantité</t>
+  </si>
+  <si>
+    <t>bo/CodeController.php</t>
+  </si>
+  <si>
+    <t>CRUD codes + génération aléatoire unique + invalidation</t>
+  </si>
+  <si>
+    <t>BO PARAMÈTRES</t>
+  </si>
+  <si>
+    <t>parametres.sql</t>
+  </si>
+  <si>
+    <t>Table parametres : id, cle, valeur, description</t>
+  </si>
+  <si>
+    <t>bo/parametres.php</t>
+  </si>
+  <si>
+    <t>Page CRUD paramètres : prix Gold, seuils IMC</t>
+  </si>
+  <si>
+    <t>bo/ParamController.php</t>
+  </si>
+  <si>
+    <t>Logique CRUD paramètres généraux en base</t>
+  </si>
+  <si>
+    <t>BASE DE DONNÉES</t>
+  </si>
+  <si>
+    <t>base.sql</t>
+  </si>
+  <si>
+    <t>Script SQL complet : CREATE TABLE, contraintes, clés étrangères</t>
+  </si>
+  <si>
+    <t>Données de test : 5 users, 15 codes, 5 régimes, 5 activités</t>
+  </si>
+  <si>
     <t>Sélection activités sportives associées + durée estimée</t>
   </si>
   <si>
-    <t>Affichage prix avec/sans remise Gold (15%)</t>
-  </si>
-  <si>
-    <t>PHP/HTML</t>
-  </si>
-  <si>
-    <t>EXPORT PDF</t>
-  </si>
-  <si>
-    <t>export_pdf.php</t>
-  </si>
-  <si>
-    <t>Intégration bibliothèque TCPDF ou DomPDF via Composer</t>
-  </si>
-  <si>
-    <t>PHP</t>
-  </si>
-  <si>
-    <t>Génération PDF : résumé régime + activités + IMC utilisateur</t>
-  </si>
-  <si>
-    <t>PORTE MONNAIE</t>
-  </si>
-  <si>
-    <t>wallet.php</t>
-  </si>
-  <si>
-    <t>Design page portefeuille : affichage solde + champ saisie code</t>
-  </si>
-  <si>
-    <t>WalletController.php</t>
-  </si>
-  <si>
-    <t>Vérification code via AJAX : validation, crédit solde, marque utilisé</t>
-  </si>
-  <si>
-    <t>codes.sql</t>
-  </si>
-  <si>
-    <t>Table codes : id, code, montant, statut (actif/utilisé), user_id</t>
-  </si>
-  <si>
-    <t>OPTION GOLD</t>
-  </si>
-  <si>
-    <t>gold.php</t>
-  </si>
-  <si>
-    <t>Design page Gold : présentation avantages, prix, bouton achat</t>
-  </si>
-  <si>
-    <t>GoldController.php</t>
-  </si>
-  <si>
-    <t>Logique achat Gold : vérif solde suffisant, débit wallet, activation flag</t>
-  </si>
-  <si>
-    <t>Application automatique remise 15% si is_gold = 1</t>
-  </si>
-  <si>
-    <t>BO LOGIN</t>
-  </si>
-  <si>
-    <t>bo/login.php</t>
-  </si>
-  <si>
-    <t>Design page authentification back-office (formulaire simple)</t>
-  </si>
-  <si>
-    <t>bo/AdminController.php</t>
-  </si>
-  <si>
-    <t>Logique login admin : session séparée, rôle admin vérifié</t>
-  </si>
-  <si>
-    <t>BO DASHBOARD</t>
-  </si>
-  <si>
-    <t>bo/dashboard.php</t>
-  </si>
-  <si>
-    <t>Design tableau de bord : cards KPI (nb users, CA, codes validés)</t>
-  </si>
-  <si>
-    <t>Graphe Chart.js : évolution inscriptions par mois (ligne)</t>
-  </si>
-  <si>
-    <t>Graphe Chart.js : répartition objectifs utilisateurs (camembert)</t>
-  </si>
-  <si>
-    <t>bo/DashboardController.php</t>
-  </si>
-  <si>
-    <t>Requêtes SQL pour KPI et données graphes (agrégats)</t>
-  </si>
-  <si>
-    <t>PHP/SQL</t>
-  </si>
-  <si>
-    <t>BO RÉGIMES</t>
-  </si>
-  <si>
-    <t>bo/regimes.php</t>
-  </si>
-  <si>
-    <t>Liste régimes : tableau paginé avec actions éditer/supprimer</t>
-  </si>
-  <si>
-    <t>bo/regimes_form.php</t>
-  </si>
-  <si>
-    <t>Formulaire création/édition : nom, % viande, % poisson, % volaille, durée, prix, delta_poids</t>
-  </si>
-  <si>
-    <t>bo/RegimeController.php</t>
-  </si>
-  <si>
-    <t>CRUD complet régimes avec validation (somme % = 100)</t>
-  </si>
-  <si>
-    <t>regimes.sql</t>
-  </si>
-  <si>
-    <t>Table régimes : id, nom, pct_viande, pct_poisson, pct_volaille, duree_jours, prix, delta_poids_min, delta_poids_max</t>
-  </si>
-  <si>
-    <t>BO ACTIVITÉS</t>
-  </si>
-  <si>
-    <t>bo/activites.php</t>
-  </si>
-  <si>
-    <t>Liste + formulaire création/édition activité sportive</t>
-  </si>
-  <si>
-    <t>bo/ActiviteController.php</t>
-  </si>
-  <si>
-    <t>CRUD complet activités sportives</t>
-  </si>
-  <si>
-    <t>activites.sql</t>
-  </si>
-  <si>
-    <t>Table activités : id, nom, description, duree_min, calories_heure, niveau</t>
-  </si>
-  <si>
-    <t>BO CODES</t>
-  </si>
-  <si>
-    <t>bo/codes.php</t>
-  </si>
-  <si>
-    <t>Liste codes : tableau avec statut actif/utilisé + pagination</t>
-  </si>
-  <si>
-    <t>bo/codes_form.php</t>
-  </si>
-  <si>
-    <t>Formulaire génération de codes : montant, quantité à générer</t>
-  </si>
-  <si>
-    <t>bo/CodeController.php</t>
-  </si>
-  <si>
-    <t>CRUD codes + génération aléatoire unique + invalidation</t>
-  </si>
-  <si>
-    <t>BO PARAMÈTRES</t>
-  </si>
-  <si>
-    <t>bo/parametres.php</t>
-  </si>
-  <si>
-    <t>Page CRUD paramètres : prix Gold, seuils IMC (maigreur/obésité)</t>
-  </si>
-  <si>
-    <t>HTML/CSS/PHP</t>
-  </si>
-  <si>
-    <t>bo/ParamController.php</t>
-  </si>
-  <si>
-    <t>Logique CRUD paramètres généraux en base</t>
-  </si>
-  <si>
-    <t>parametres.sql</t>
-  </si>
-  <si>
-    <t>Table parametres : id, cle, valeur, description</t>
-  </si>
-  <si>
-    <t>BASE DE DONNÉES</t>
-  </si>
-  <si>
-    <t>base.sql</t>
-  </si>
-  <si>
-    <t>Script SQL complet : CREATE TABLE, contraintes, clés étrangères</t>
-  </si>
-  <si>
-    <t>Données de test : 5 users, 15 codes, 5 régimes, 5 activités</t>
-  </si>
-  <si>
-    <t>NAVIGATION</t>
-  </si>
-  <si>
-    <t>layout/navbar.php</t>
-  </si>
-  <si>
-    <t>Navbar front responsive : logo, liens, état connecté/déconnecté</t>
-  </si>
-  <si>
-    <t>layout/sidebar_bo.php</t>
-  </si>
-  <si>
-    <t>Sidebar back-office responsive avec liens vers toutes les sections</t>
-  </si>
-  <si>
     <t>TESTS &amp; LIVRAISON</t>
   </si>
   <si>
     <t>—</t>
   </si>
   <si>
-    <t>Tests manuels complet front-office (inscription → achat → export PDF)</t>
+    <t>Tests manuels front-office : inscription → objectif → achat → export PDF</t>
   </si>
   <si>
     <t>Tests</t>
   </si>
   <si>
-    <t>Tests manuels complet back-office (CRUD, stats, codes)</t>
+    <t>Tests manuels back-office : CRUD régimes, activités, codes, stats</t>
   </si>
   <si>
     <t>README.md</t>
@@ -420,7 +414,7 @@
     <t>gitlab</t>
   </si>
   <si>
-    <t>Revue finale du code, merge branches → main, tag de version</t>
+    <t>Revue finale du code, merge branches → main, tag de version livraison</t>
   </si>
   <si>
     <t>RÉSUMÉ GLOBAL DU PROJET</t>
@@ -457,9 +451,6 @@
   </si>
   <si>
     <t>TOTAL</t>
-  </si>
-  <si>
-    <t>SUIVI PAR TYPE DE TÂCHE</t>
   </si>
   <si>
     <t>TABLEAU CROISÉ : ESTIMATION (min) PAR MODULE × PERSONNE</t>
@@ -487,7 +478,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="27">
+  <fonts count="19">
     <font>
       <sz val="11.0"/>
       <color theme="1"/>
@@ -508,7 +499,7 @@
     <font>
       <b/>
       <sz val="9.0"/>
-      <color rgb="FF8E24AA"/>
+      <color rgb="FF2471B0"/>
       <name val="Arial"/>
     </font>
     <font>
@@ -531,7 +522,7 @@
     <font>
       <b/>
       <sz val="9.0"/>
-      <color rgb="FF2471B0"/>
+      <color rgb="FF8E24AA"/>
       <name val="Arial"/>
     </font>
     <font>
@@ -572,8 +563,9 @@
       <name val="Arial"/>
     </font>
     <font>
+      <b/>
       <sz val="9.0"/>
-      <color rgb="FFE74C3C"/>
+      <color rgb="FF1F2D3D"/>
       <name val="Arial"/>
     </font>
     <font>
@@ -583,56 +575,12 @@
     </font>
     <font>
       <sz val="9.0"/>
-      <color rgb="FF27AE60"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9.0"/>
-      <color rgb="FFE67E22"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="9.0"/>
-      <color rgb="FFE67E22"/>
+      <color rgb="FF1A7A4A"/>
       <name val="Arial"/>
     </font>
     <font>
       <sz val="9.0"/>
       <color rgb="FF8E24AA"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="9.0"/>
-      <color rgb="FF1A7A4A"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9.0"/>
-      <color rgb="FF555555"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="9.0"/>
-      <color rgb="FF555555"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9.0"/>
-      <color rgb="FF7F8C8D"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="9.0"/>
-      <color rgb="FF7F8C8D"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9.0"/>
-      <color rgb="FF1F2D3D"/>
       <name val="Arial"/>
     </font>
   </fonts>
@@ -730,7 +678,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="73">
+  <cellXfs count="51">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -796,7 +744,7 @@
     <xf borderId="1" fillId="6" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="3" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="1" fillId="3" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -805,7 +753,7 @@
     <xf borderId="1" fillId="3" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="3" fontId="3" numFmtId="9" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="3" fontId="7" numFmtId="9" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="1" fillId="3" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -814,13 +762,13 @@
     <xf borderId="2" fillId="2" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="5" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="5" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="1" fillId="5" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="5" fontId="7" numFmtId="9" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="5" fontId="3" numFmtId="9" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="1" fillId="3" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -832,10 +780,10 @@
     <xf borderId="1" fillId="3" fontId="6" numFmtId="9" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="5" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="5" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="5" fontId="3" numFmtId="9" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="5" fontId="7" numFmtId="9" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="1" fillId="7" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
@@ -847,103 +795,37 @@
     <xf borderId="1" fillId="7" fontId="1" numFmtId="9" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="3" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="1" fillId="3" fontId="15" numFmtId="9" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="1" fillId="5" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="1" fillId="5" fontId="16" numFmtId="9" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="1" fillId="3" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="1" fillId="3" fontId="17" numFmtId="9" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="1" fillId="5" fontId="18" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="1" fillId="5" fontId="19" numFmtId="9" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="1" fillId="3" fontId="18" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="1" fillId="3" fontId="19" numFmtId="9" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="1" fillId="5" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="1" fillId="5" fontId="20" numFmtId="9" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="1" fillId="3" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="1" fillId="3" fontId="21" numFmtId="9" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="1" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="1" fillId="3" fontId="20" numFmtId="9" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="1" fillId="5" fontId="22" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="1" fillId="5" fontId="23" numFmtId="9" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="1" fillId="3" fontId="24" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="1" fillId="3" fontId="25" numFmtId="9" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="1" fillId="5" fontId="24" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="1" fillId="5" fontId="25" numFmtId="9" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="1" fillId="5" fontId="26" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="5" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="1" fillId="5" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="5" fontId="21" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="5" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="5" fontId="20" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="5" fontId="18" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="1" fillId="5" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="3" fontId="26" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="3" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="1" fillId="3" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="3" fontId="21" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="3" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="3" fontId="20" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="3" fontId="18" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="1" fillId="5" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="3" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
   </cellXfs>
@@ -1279,21 +1161,21 @@
         <v>14</v>
       </c>
       <c r="F2" s="2">
-        <v>90.0</v>
+        <v>20.0</v>
       </c>
       <c r="G2" s="5">
         <v>0.0</v>
       </c>
       <c r="H2" s="6">
-        <f t="shared" ref="H2:H55" si="1">MAX(0,F2-G2)</f>
-        <v>90</v>
+        <f t="shared" ref="H2:H53" si="1">MAX(0,F2-G2)</f>
+        <v>20</v>
       </c>
       <c r="I2" s="7">
-        <f t="shared" ref="I2:I55" si="2">IFERROR(MIN(1,G2/F2),0)</f>
+        <f t="shared" ref="I2:I53" si="2">IFERROR(MIN(1,G2/F2),0)</f>
         <v>0</v>
       </c>
       <c r="J2" s="8" t="str">
-        <f t="shared" ref="J2:J55" si="3">IF(G2=0,"À FAIRE",IF(I2&gt;=1,"OK","EN COURS"))</f>
+        <f t="shared" ref="J2:J53" si="3">IF(G2=0,"À FAIRE",IF(I2&gt;=1,"OK","EN COURS"))</f>
         <v>À FAIRE</v>
       </c>
     </row>
@@ -1302,26 +1184,26 @@
         <v>10</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E3" s="11" t="s">
         <v>14</v>
       </c>
       <c r="F3" s="9">
-        <v>45.0</v>
+        <v>60.0</v>
       </c>
       <c r="G3" s="5">
         <v>0.0</v>
       </c>
       <c r="H3" s="12">
         <f t="shared" si="1"/>
-        <v>45</v>
+        <v>60</v>
       </c>
       <c r="I3" s="13">
         <f t="shared" si="2"/>
@@ -1337,26 +1219,26 @@
         <v>10</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>18</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E4" s="15" t="s">
         <v>19</v>
       </c>
+      <c r="E4" s="4" t="s">
+        <v>14</v>
+      </c>
       <c r="F4" s="2">
-        <v>60.0</v>
+        <v>40.0</v>
       </c>
       <c r="G4" s="5">
         <v>0.0</v>
       </c>
       <c r="H4" s="6">
         <f t="shared" si="1"/>
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="I4" s="7">
         <f t="shared" si="2"/>
@@ -1372,26 +1254,26 @@
         <v>10</v>
       </c>
       <c r="B5" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="D5" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="C5" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="D5" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="E5" s="16" t="s">
-        <v>19</v>
+      <c r="E5" s="11" t="s">
+        <v>14</v>
       </c>
       <c r="F5" s="9">
-        <v>60.0</v>
+        <v>50.0</v>
       </c>
       <c r="G5" s="5">
         <v>0.0</v>
       </c>
       <c r="H5" s="12">
         <f t="shared" si="1"/>
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="I5" s="13">
         <f t="shared" si="2"/>
@@ -1407,26 +1289,26 @@
         <v>10</v>
       </c>
       <c r="B6" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C6" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="D6" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="D6" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="E6" s="17" t="s">
-        <v>25</v>
+      <c r="E6" s="4" t="s">
+        <v>14</v>
       </c>
       <c r="F6" s="2">
-        <v>90.0</v>
+        <v>50.0</v>
       </c>
       <c r="G6" s="5">
         <v>0.0</v>
       </c>
       <c r="H6" s="6">
         <f t="shared" si="1"/>
-        <v>90</v>
+        <v>50</v>
       </c>
       <c r="I6" s="7">
         <f t="shared" si="2"/>
@@ -1442,26 +1324,26 @@
         <v>10</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C7" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="D7" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="D7" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="E7" s="18" t="s">
-        <v>25</v>
+      <c r="E7" s="11" t="s">
+        <v>14</v>
       </c>
       <c r="F7" s="9">
-        <v>30.0</v>
+        <v>90.0</v>
       </c>
       <c r="G7" s="5">
         <v>0.0</v>
       </c>
       <c r="H7" s="12">
         <f t="shared" si="1"/>
-        <v>30</v>
+        <v>90</v>
       </c>
       <c r="I7" s="13">
         <f t="shared" si="2"/>
@@ -1474,29 +1356,29 @@
     </row>
     <row r="8" ht="21.75" customHeight="1">
       <c r="A8" s="2" t="s">
-        <v>10</v>
+        <v>27</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="E8" s="17" t="s">
-        <v>25</v>
+        <v>17</v>
+      </c>
+      <c r="E8" s="15" t="s">
+        <v>30</v>
       </c>
       <c r="F8" s="2">
-        <v>20.0</v>
+        <v>40.0</v>
       </c>
       <c r="G8" s="5">
         <v>0.0</v>
       </c>
       <c r="H8" s="6">
         <f t="shared" si="1"/>
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="I8" s="7">
         <f t="shared" si="2"/>
@@ -1509,29 +1391,29 @@
     </row>
     <row r="9" ht="21.75" customHeight="1">
       <c r="A9" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="B9" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="C9" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="D9" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E9" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="B9" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="C9" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="D9" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="E9" s="11" t="s">
-        <v>14</v>
-      </c>
       <c r="F9" s="9">
-        <v>45.0</v>
+        <v>70.0</v>
       </c>
       <c r="G9" s="5">
         <v>0.0</v>
       </c>
       <c r="H9" s="12">
         <f t="shared" si="1"/>
-        <v>45</v>
+        <v>70</v>
       </c>
       <c r="I9" s="13">
         <f t="shared" si="2"/>
@@ -1544,29 +1426,29 @@
     </row>
     <row r="10" ht="21.75" customHeight="1">
       <c r="A10" s="2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>22</v>
+        <v>33</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="E10" s="17" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="F10" s="2">
-        <v>45.0</v>
+        <v>60.0</v>
       </c>
       <c r="G10" s="5">
         <v>0.0</v>
       </c>
       <c r="H10" s="6">
         <f t="shared" si="1"/>
-        <v>45</v>
+        <v>60</v>
       </c>
       <c r="I10" s="7">
         <f t="shared" si="2"/>
@@ -1579,29 +1461,29 @@
     </row>
     <row r="11" ht="21.75" customHeight="1">
       <c r="A11" s="9" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>22</v>
+        <v>36</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>24</v>
+        <v>38</v>
       </c>
       <c r="E11" s="18" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="F11" s="9">
-        <v>15.0</v>
+        <v>60.0</v>
       </c>
       <c r="G11" s="5">
         <v>0.0</v>
       </c>
       <c r="H11" s="12">
         <f t="shared" si="1"/>
-        <v>15</v>
+        <v>60</v>
       </c>
       <c r="I11" s="13">
         <f t="shared" si="2"/>
@@ -1614,29 +1496,29 @@
     </row>
     <row r="12" ht="21.75" customHeight="1">
       <c r="A12" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E12" s="15" t="s">
         <v>30</v>
       </c>
-      <c r="B12" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="E12" s="17" t="s">
-        <v>25</v>
-      </c>
       <c r="F12" s="2">
-        <v>30.0</v>
+        <v>55.0</v>
       </c>
       <c r="G12" s="5">
         <v>0.0</v>
       </c>
       <c r="H12" s="6">
         <f t="shared" si="1"/>
-        <v>30</v>
+        <v>55</v>
       </c>
       <c r="I12" s="7">
         <f t="shared" si="2"/>
@@ -1649,29 +1531,29 @@
     </row>
     <row r="13" ht="21.75" customHeight="1">
       <c r="A13" s="9" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="E13" s="11" t="s">
-        <v>14</v>
+        <v>26</v>
+      </c>
+      <c r="E13" s="16" t="s">
+        <v>30</v>
       </c>
       <c r="F13" s="9">
-        <v>60.0</v>
+        <v>35.0</v>
       </c>
       <c r="G13" s="5">
         <v>0.0</v>
       </c>
       <c r="H13" s="12">
         <f t="shared" si="1"/>
-        <v>60</v>
+        <v>35</v>
       </c>
       <c r="I13" s="13">
         <f t="shared" si="2"/>
@@ -1684,29 +1566,29 @@
     </row>
     <row r="14" ht="21.75" customHeight="1">
       <c r="A14" s="2" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>41</v>
+        <v>17</v>
       </c>
       <c r="E14" s="17" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="F14" s="2">
-        <v>60.0</v>
+        <v>80.0</v>
       </c>
       <c r="G14" s="5">
         <v>0.0</v>
       </c>
       <c r="H14" s="6">
         <f t="shared" si="1"/>
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="I14" s="7">
         <f t="shared" si="2"/>
@@ -1719,29 +1601,29 @@
     </row>
     <row r="15" ht="21.75" customHeight="1">
       <c r="A15" s="9" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="E15" s="11" t="s">
-        <v>14</v>
+        <v>26</v>
+      </c>
+      <c r="E15" s="18" t="s">
+        <v>35</v>
       </c>
       <c r="F15" s="9">
-        <v>60.0</v>
+        <v>120.0</v>
       </c>
       <c r="G15" s="5">
         <v>0.0</v>
       </c>
       <c r="H15" s="12">
         <f t="shared" si="1"/>
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="I15" s="13">
         <f t="shared" si="2"/>
@@ -1754,29 +1636,29 @@
     </row>
     <row r="16" ht="21.75" customHeight="1">
       <c r="A16" s="2" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>45</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>24</v>
+        <v>50</v>
       </c>
       <c r="E16" s="17" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="F16" s="2">
-        <v>30.0</v>
+        <v>40.0</v>
       </c>
       <c r="G16" s="5">
         <v>0.0</v>
       </c>
       <c r="H16" s="6">
         <f t="shared" si="1"/>
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="I16" s="7">
         <f t="shared" si="2"/>
@@ -1789,29 +1671,29 @@
     </row>
     <row r="17" ht="21.75" customHeight="1">
       <c r="A17" s="9" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="D17" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="E17" s="11" t="s">
-        <v>14</v>
+        <v>54</v>
+      </c>
+      <c r="E17" s="16" t="s">
+        <v>30</v>
       </c>
       <c r="F17" s="9">
-        <v>90.0</v>
+        <v>45.0</v>
       </c>
       <c r="G17" s="5">
         <v>0.0</v>
       </c>
       <c r="H17" s="12">
         <f t="shared" si="1"/>
-        <v>90</v>
+        <v>45</v>
       </c>
       <c r="I17" s="13">
         <f t="shared" si="2"/>
@@ -1824,29 +1706,29 @@
     </row>
     <row r="18" ht="21.75" customHeight="1">
       <c r="A18" s="2" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="E18" s="17" t="s">
-        <v>25</v>
+        <v>54</v>
+      </c>
+      <c r="E18" s="15" t="s">
+        <v>30</v>
       </c>
       <c r="F18" s="2">
-        <v>120.0</v>
+        <v>90.0</v>
       </c>
       <c r="G18" s="5">
         <v>0.0</v>
       </c>
       <c r="H18" s="6">
         <f t="shared" si="1"/>
-        <v>120</v>
+        <v>90</v>
       </c>
       <c r="I18" s="7">
         <f t="shared" si="2"/>
@@ -1859,29 +1741,29 @@
     </row>
     <row r="19" ht="21.75" customHeight="1">
       <c r="A19" s="9" t="s">
-        <v>47</v>
+        <v>56</v>
       </c>
       <c r="B19" s="10" t="s">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="D19" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="E19" s="18" t="s">
-        <v>25</v>
+        <v>17</v>
+      </c>
+      <c r="E19" s="11" t="s">
+        <v>14</v>
       </c>
       <c r="F19" s="9">
-        <v>60.0</v>
+        <v>40.0</v>
       </c>
       <c r="G19" s="5">
         <v>0.0</v>
       </c>
       <c r="H19" s="12">
         <f t="shared" si="1"/>
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="I19" s="13">
         <f t="shared" si="2"/>
@@ -1894,29 +1776,29 @@
     </row>
     <row r="20" ht="21.75" customHeight="1">
       <c r="A20" s="2" t="s">
-        <v>47</v>
+        <v>56</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>48</v>
+        <v>59</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="E20" s="15" t="s">
-        <v>19</v>
+        <v>38</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>14</v>
       </c>
       <c r="F20" s="2">
-        <v>45.0</v>
+        <v>70.0</v>
       </c>
       <c r="G20" s="5">
         <v>0.0</v>
       </c>
       <c r="H20" s="6">
         <f t="shared" si="1"/>
-        <v>45</v>
+        <v>70</v>
       </c>
       <c r="I20" s="7">
         <f t="shared" si="2"/>
@@ -1929,29 +1811,29 @@
     </row>
     <row r="21" ht="21.75" customHeight="1">
       <c r="A21" s="9" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B21" s="10" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="D21" s="9" t="s">
-        <v>58</v>
-      </c>
-      <c r="E21" s="16" t="s">
-        <v>19</v>
+        <v>13</v>
+      </c>
+      <c r="E21" s="11" t="s">
+        <v>14</v>
       </c>
       <c r="F21" s="9">
-        <v>45.0</v>
+        <v>15.0</v>
       </c>
       <c r="G21" s="5">
         <v>0.0</v>
       </c>
       <c r="H21" s="12">
         <f t="shared" si="1"/>
-        <v>45</v>
+        <v>15</v>
       </c>
       <c r="I21" s="13">
         <f t="shared" si="2"/>
@@ -1964,29 +1846,29 @@
     </row>
     <row r="22" ht="21.75" customHeight="1">
       <c r="A22" s="2" t="s">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>56</v>
+        <v>64</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>58</v>
+        <v>17</v>
       </c>
       <c r="E22" s="15" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="F22" s="2">
-        <v>90.0</v>
+        <v>45.0</v>
       </c>
       <c r="G22" s="5">
         <v>0.0</v>
       </c>
       <c r="H22" s="6">
         <f t="shared" si="1"/>
-        <v>90</v>
+        <v>45</v>
       </c>
       <c r="I22" s="7">
         <f t="shared" si="2"/>
@@ -1999,29 +1881,29 @@
     </row>
     <row r="23" ht="21.75" customHeight="1">
       <c r="A23" s="9" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="B23" s="10" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="D23" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="E23" s="11" t="s">
-        <v>14</v>
+        <v>26</v>
+      </c>
+      <c r="E23" s="16" t="s">
+        <v>30</v>
       </c>
       <c r="F23" s="9">
-        <v>45.0</v>
+        <v>60.0</v>
       </c>
       <c r="G23" s="5">
         <v>0.0</v>
       </c>
       <c r="H23" s="12">
         <f t="shared" si="1"/>
-        <v>45</v>
+        <v>60</v>
       </c>
       <c r="I23" s="13">
         <f t="shared" si="2"/>
@@ -2034,29 +1916,29 @@
     </row>
     <row r="24" ht="21.75" customHeight="1">
       <c r="A24" s="2" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="E24" s="17" t="s">
-        <v>25</v>
+        <v>26</v>
+      </c>
+      <c r="E24" s="4" t="s">
+        <v>14</v>
       </c>
       <c r="F24" s="2">
-        <v>75.0</v>
+        <v>30.0</v>
       </c>
       <c r="G24" s="5">
         <v>0.0</v>
       </c>
       <c r="H24" s="6">
         <f t="shared" si="1"/>
-        <v>75</v>
+        <v>30</v>
       </c>
       <c r="I24" s="7">
         <f t="shared" si="2"/>
@@ -2069,29 +1951,29 @@
     </row>
     <row r="25" ht="21.75" customHeight="1">
       <c r="A25" s="9" t="s">
-        <v>60</v>
+        <v>69</v>
       </c>
       <c r="B25" s="10" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="C25" s="10" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="D25" s="9" t="s">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="E25" s="18" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="F25" s="9">
-        <v>15.0</v>
+        <v>55.0</v>
       </c>
       <c r="G25" s="5">
         <v>0.0</v>
       </c>
       <c r="H25" s="12">
         <f t="shared" si="1"/>
-        <v>15</v>
+        <v>55</v>
       </c>
       <c r="I25" s="13">
         <f t="shared" si="2"/>
@@ -2104,29 +1986,29 @@
     </row>
     <row r="26" ht="21.75" customHeight="1">
       <c r="A26" s="2" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E26" s="4" t="s">
-        <v>14</v>
+        <v>17</v>
+      </c>
+      <c r="E26" s="17" t="s">
+        <v>35</v>
       </c>
       <c r="F26" s="2">
-        <v>45.0</v>
+        <v>50.0</v>
       </c>
       <c r="G26" s="5">
         <v>0.0</v>
       </c>
       <c r="H26" s="6">
         <f t="shared" si="1"/>
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="I26" s="7">
         <f t="shared" si="2"/>
@@ -2139,29 +2021,29 @@
     </row>
     <row r="27" ht="21.75" customHeight="1">
       <c r="A27" s="9" t="s">
-        <v>67</v>
+        <v>74</v>
       </c>
       <c r="B27" s="10" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="D27" s="9" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="E27" s="16" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="F27" s="9">
-        <v>60.0</v>
+        <v>50.0</v>
       </c>
       <c r="G27" s="5">
         <v>0.0</v>
       </c>
       <c r="H27" s="12">
         <f t="shared" si="1"/>
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="I27" s="13">
         <f t="shared" si="2"/>
@@ -2174,19 +2056,19 @@
     </row>
     <row r="28" ht="21.75" customHeight="1">
       <c r="A28" s="2" t="s">
-        <v>67</v>
+        <v>74</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="E28" s="17" t="s">
-        <v>25</v>
+        <v>26</v>
+      </c>
+      <c r="E28" s="15" t="s">
+        <v>30</v>
       </c>
       <c r="F28" s="2">
         <v>30.0</v>
@@ -2209,29 +2091,29 @@
     </row>
     <row r="29" ht="21.75" customHeight="1">
       <c r="A29" s="9" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="B29" s="10" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="D29" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="E29" s="11" t="s">
-        <v>14</v>
+        <v>17</v>
+      </c>
+      <c r="E29" s="18" t="s">
+        <v>35</v>
       </c>
       <c r="F29" s="9">
-        <v>30.0</v>
+        <v>80.0</v>
       </c>
       <c r="G29" s="5">
         <v>0.0</v>
       </c>
       <c r="H29" s="12">
         <f t="shared" si="1"/>
-        <v>30</v>
+        <v>80</v>
       </c>
       <c r="I29" s="13">
         <f t="shared" si="2"/>
@@ -2244,29 +2126,29 @@
     </row>
     <row r="30" ht="21.75" customHeight="1">
       <c r="A30" s="2" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="E30" s="17" t="s">
-        <v>25</v>
+        <v>19</v>
+      </c>
+      <c r="E30" s="4" t="s">
+        <v>14</v>
       </c>
       <c r="F30" s="2">
-        <v>40.0</v>
+        <v>75.0</v>
       </c>
       <c r="G30" s="5">
         <v>0.0</v>
       </c>
       <c r="H30" s="6">
         <f t="shared" si="1"/>
-        <v>40</v>
+        <v>75</v>
       </c>
       <c r="I30" s="7">
         <f t="shared" si="2"/>
@@ -2279,29 +2161,29 @@
     </row>
     <row r="31" ht="21.75" customHeight="1">
       <c r="A31" s="9" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B31" s="10" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C31" s="10" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="D31" s="9" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="E31" s="16" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="F31" s="9">
-        <v>90.0</v>
+        <v>60.0</v>
       </c>
       <c r="G31" s="5">
         <v>0.0</v>
       </c>
       <c r="H31" s="12">
         <f t="shared" si="1"/>
-        <v>90</v>
+        <v>60</v>
       </c>
       <c r="I31" s="13">
         <f t="shared" si="2"/>
@@ -2314,29 +2196,29 @@
     </row>
     <row r="32" ht="21.75" customHeight="1">
       <c r="A32" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="E32" s="15" t="s">
-        <v>19</v>
+        <v>86</v>
+      </c>
+      <c r="E32" s="17" t="s">
+        <v>35</v>
       </c>
       <c r="F32" s="2">
-        <v>75.0</v>
+        <v>55.0</v>
       </c>
       <c r="G32" s="5">
         <v>0.0</v>
       </c>
       <c r="H32" s="6">
         <f t="shared" si="1"/>
-        <v>75</v>
+        <v>55</v>
       </c>
       <c r="I32" s="7">
         <f t="shared" si="2"/>
@@ -2349,29 +2231,29 @@
     </row>
     <row r="33" ht="21.75" customHeight="1">
       <c r="A33" s="9" t="s">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="B33" s="10" t="s">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="C33" s="10" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="D33" s="9" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="E33" s="11" t="s">
         <v>14</v>
       </c>
       <c r="F33" s="9">
-        <v>60.0</v>
+        <v>20.0</v>
       </c>
       <c r="G33" s="5">
         <v>0.0</v>
       </c>
       <c r="H33" s="12">
         <f t="shared" si="1"/>
-        <v>60</v>
+        <v>20</v>
       </c>
       <c r="I33" s="13">
         <f t="shared" si="2"/>
@@ -2384,29 +2266,29 @@
     </row>
     <row r="34" ht="21.75" customHeight="1">
       <c r="A34" s="2" t="s">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>85</v>
+        <v>17</v>
       </c>
       <c r="E34" s="17" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="F34" s="2">
-        <v>60.0</v>
+        <v>55.0</v>
       </c>
       <c r="G34" s="5">
         <v>0.0</v>
       </c>
       <c r="H34" s="6">
         <f t="shared" si="1"/>
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="I34" s="7">
         <f t="shared" si="2"/>
@@ -2419,29 +2301,29 @@
     </row>
     <row r="35" ht="21.75" customHeight="1">
       <c r="A35" s="9" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B35" s="10" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="C35" s="10" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="D35" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="E35" s="11" t="s">
-        <v>14</v>
+        <v>17</v>
+      </c>
+      <c r="E35" s="16" t="s">
+        <v>30</v>
       </c>
       <c r="F35" s="9">
-        <v>60.0</v>
+        <v>65.0</v>
       </c>
       <c r="G35" s="5">
         <v>0.0</v>
       </c>
       <c r="H35" s="12">
         <f t="shared" si="1"/>
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="I35" s="13">
         <f t="shared" si="2"/>
@@ -2454,29 +2336,29 @@
     </row>
     <row r="36" ht="21.75" customHeight="1">
       <c r="A36" s="2" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E36" s="15" t="s">
-        <v>19</v>
+        <v>26</v>
+      </c>
+      <c r="E36" s="4" t="s">
+        <v>14</v>
       </c>
       <c r="F36" s="2">
-        <v>75.0</v>
+        <v>85.0</v>
       </c>
       <c r="G36" s="5">
         <v>0.0</v>
       </c>
       <c r="H36" s="6">
         <f t="shared" si="1"/>
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="I36" s="7">
         <f t="shared" si="2"/>
@@ -2489,29 +2371,29 @@
     </row>
     <row r="37" ht="21.75" customHeight="1">
       <c r="A37" s="9" t="s">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="B37" s="10" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="C37" s="10" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="D37" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="E37" s="18" t="s">
-        <v>25</v>
+        <v>13</v>
+      </c>
+      <c r="E37" s="16" t="s">
+        <v>30</v>
       </c>
       <c r="F37" s="9">
-        <v>90.0</v>
+        <v>15.0</v>
       </c>
       <c r="G37" s="5">
         <v>0.0</v>
       </c>
       <c r="H37" s="12">
         <f t="shared" si="1"/>
-        <v>90</v>
+        <v>15</v>
       </c>
       <c r="I37" s="13">
         <f t="shared" si="2"/>
@@ -2524,29 +2406,29 @@
     </row>
     <row r="38" ht="21.75" customHeight="1">
       <c r="A38" s="2" t="s">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="E38" s="17" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="F38" s="2">
-        <v>20.0</v>
+        <v>50.0</v>
       </c>
       <c r="G38" s="5">
         <v>0.0</v>
       </c>
       <c r="H38" s="6">
         <f t="shared" si="1"/>
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="I38" s="7">
         <f t="shared" si="2"/>
@@ -2559,29 +2441,29 @@
     </row>
     <row r="39" ht="21.75" customHeight="1">
       <c r="A39" s="9" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B39" s="10" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="C39" s="10" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="D39" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="E39" s="11" t="s">
-        <v>14</v>
+        <v>17</v>
+      </c>
+      <c r="E39" s="18" t="s">
+        <v>35</v>
       </c>
       <c r="F39" s="9">
-        <v>60.0</v>
+        <v>40.0</v>
       </c>
       <c r="G39" s="5">
         <v>0.0</v>
       </c>
       <c r="H39" s="12">
         <f t="shared" si="1"/>
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="I39" s="13">
         <f t="shared" si="2"/>
@@ -2594,19 +2476,19 @@
     </row>
     <row r="40" ht="21.75" customHeight="1">
       <c r="A40" s="2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="E40" s="17" t="s">
-        <v>25</v>
+        <v>26</v>
+      </c>
+      <c r="E40" s="15" t="s">
+        <v>30</v>
       </c>
       <c r="F40" s="2">
         <v>60.0</v>
@@ -2629,29 +2511,29 @@
     </row>
     <row r="41" ht="21.75" customHeight="1">
       <c r="A41" s="9" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="B41" s="10" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="C41" s="10" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="D41" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="E41" s="18" t="s">
-        <v>25</v>
+        <v>17</v>
+      </c>
+      <c r="E41" s="11" t="s">
+        <v>14</v>
       </c>
       <c r="F41" s="9">
-        <v>15.0</v>
+        <v>40.0</v>
       </c>
       <c r="G41" s="5">
         <v>0.0</v>
       </c>
       <c r="H41" s="12">
         <f t="shared" si="1"/>
-        <v>15</v>
+        <v>40</v>
       </c>
       <c r="I41" s="13">
         <f t="shared" si="2"/>
@@ -2664,29 +2546,29 @@
     </row>
     <row r="42" ht="21.75" customHeight="1">
       <c r="A42" s="2" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E42" s="15" t="s">
-        <v>19</v>
+        <v>17</v>
+      </c>
+      <c r="E42" s="4" t="s">
+        <v>14</v>
       </c>
       <c r="F42" s="2">
-        <v>45.0</v>
+        <v>40.0</v>
       </c>
       <c r="G42" s="5">
         <v>0.0</v>
       </c>
       <c r="H42" s="6">
         <f t="shared" si="1"/>
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="I42" s="7">
         <f t="shared" si="2"/>
@@ -2699,29 +2581,29 @@
     </row>
     <row r="43" ht="21.75" customHeight="1">
       <c r="A43" s="9" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="B43" s="10" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="C43" s="10" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="D43" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="E43" s="16" t="s">
-        <v>19</v>
+        <v>26</v>
+      </c>
+      <c r="E43" s="11" t="s">
+        <v>14</v>
       </c>
       <c r="F43" s="9">
-        <v>45.0</v>
+        <v>70.0</v>
       </c>
       <c r="G43" s="5">
         <v>0.0</v>
       </c>
       <c r="H43" s="12">
         <f t="shared" si="1"/>
-        <v>45</v>
+        <v>70</v>
       </c>
       <c r="I43" s="13">
         <f t="shared" si="2"/>
@@ -2734,29 +2616,29 @@
     </row>
     <row r="44" ht="21.75" customHeight="1">
       <c r="A44" s="2" t="s">
-        <v>102</v>
+        <v>112</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="E44" s="17" t="s">
-        <v>25</v>
+        <v>13</v>
+      </c>
+      <c r="E44" s="15" t="s">
+        <v>30</v>
       </c>
       <c r="F44" s="2">
-        <v>75.0</v>
+        <v>10.0</v>
       </c>
       <c r="G44" s="5">
         <v>0.0</v>
       </c>
       <c r="H44" s="6">
         <f t="shared" si="1"/>
-        <v>75</v>
+        <v>10</v>
       </c>
       <c r="I44" s="7">
         <f t="shared" si="2"/>
@@ -2769,29 +2651,29 @@
     </row>
     <row r="45" ht="21.75" customHeight="1">
       <c r="A45" s="9" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="B45" s="10" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="C45" s="10" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="D45" s="9" t="s">
-        <v>112</v>
-      </c>
-      <c r="E45" s="16" t="s">
-        <v>19</v>
+        <v>17</v>
+      </c>
+      <c r="E45" s="18" t="s">
+        <v>35</v>
       </c>
       <c r="F45" s="9">
-        <v>60.0</v>
+        <v>50.0</v>
       </c>
       <c r="G45" s="5">
         <v>0.0</v>
       </c>
       <c r="H45" s="12">
         <f t="shared" si="1"/>
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="I45" s="13">
         <f t="shared" si="2"/>
@@ -2804,29 +2686,29 @@
     </row>
     <row r="46" ht="21.75" customHeight="1">
       <c r="A46" s="2" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E46" s="17" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="F46" s="2">
-        <v>45.0</v>
+        <v>40.0</v>
       </c>
       <c r="G46" s="5">
         <v>0.0</v>
       </c>
       <c r="H46" s="6">
         <f t="shared" si="1"/>
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="I46" s="7">
         <f t="shared" si="2"/>
@@ -2839,29 +2721,29 @@
     </row>
     <row r="47" ht="21.75" customHeight="1">
       <c r="A47" s="9" t="s">
-        <v>109</v>
+        <v>119</v>
       </c>
       <c r="B47" s="10" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="C47" s="10" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="D47" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="E47" s="18" t="s">
-        <v>25</v>
+        <v>13</v>
+      </c>
+      <c r="E47" s="11" t="s">
+        <v>14</v>
       </c>
       <c r="F47" s="9">
-        <v>10.0</v>
+        <v>45.0</v>
       </c>
       <c r="G47" s="5">
         <v>0.0</v>
       </c>
       <c r="H47" s="12">
         <f t="shared" si="1"/>
-        <v>10</v>
+        <v>45</v>
       </c>
       <c r="I47" s="13">
         <f t="shared" si="2"/>
@@ -2874,29 +2756,29 @@
     </row>
     <row r="48" ht="21.75" customHeight="1">
       <c r="A48" s="2" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="E48" s="17" t="s">
-        <v>25</v>
+        <v>13</v>
+      </c>
+      <c r="E48" s="15" t="s">
+        <v>30</v>
       </c>
       <c r="F48" s="2">
-        <v>45.0</v>
+        <v>55.0</v>
       </c>
       <c r="G48" s="5">
         <v>0.0</v>
       </c>
       <c r="H48" s="6">
         <f t="shared" si="1"/>
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="I48" s="7">
         <f t="shared" si="2"/>
@@ -2909,29 +2791,29 @@
     </row>
     <row r="49" ht="21.75" customHeight="1">
       <c r="A49" s="9" t="s">
-        <v>117</v>
+        <v>44</v>
       </c>
       <c r="B49" s="10" t="s">
-        <v>118</v>
+        <v>47</v>
       </c>
       <c r="C49" s="10" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="D49" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="E49" s="16" t="s">
-        <v>19</v>
+        <v>26</v>
+      </c>
+      <c r="E49" s="11" t="s">
+        <v>14</v>
       </c>
       <c r="F49" s="9">
-        <v>60.0</v>
+        <v>55.0</v>
       </c>
       <c r="G49" s="5">
         <v>0.0</v>
       </c>
       <c r="H49" s="12">
         <f t="shared" si="1"/>
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="I49" s="13">
         <f t="shared" si="2"/>
@@ -2944,19 +2826,19 @@
     </row>
     <row r="50" ht="21.75" customHeight="1">
       <c r="A50" s="2" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E50" s="4" t="s">
-        <v>14</v>
+        <v>127</v>
+      </c>
+      <c r="E50" s="15" t="s">
+        <v>30</v>
       </c>
       <c r="F50" s="2">
         <v>60.0</v>
@@ -2979,29 +2861,29 @@
     </row>
     <row r="51" ht="21.75" customHeight="1">
       <c r="A51" s="9" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="B51" s="10" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C51" s="10" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="D51" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="E51" s="11" t="s">
-        <v>14</v>
+        <v>127</v>
+      </c>
+      <c r="E51" s="18" t="s">
+        <v>35</v>
       </c>
       <c r="F51" s="9">
-        <v>60.0</v>
+        <v>50.0</v>
       </c>
       <c r="G51" s="5">
         <v>0.0</v>
       </c>
       <c r="H51" s="12">
         <f t="shared" si="1"/>
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="I51" s="13">
         <f t="shared" si="2"/>
@@ -3014,29 +2896,29 @@
     </row>
     <row r="52" ht="21.75" customHeight="1">
       <c r="A52" s="2" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>129</v>
-      </c>
-      <c r="E52" s="15" t="s">
-        <v>19</v>
+        <v>131</v>
+      </c>
+      <c r="E52" s="4" t="s">
+        <v>14</v>
       </c>
       <c r="F52" s="2">
-        <v>60.0</v>
+        <v>30.0</v>
       </c>
       <c r="G52" s="5">
         <v>0.0</v>
       </c>
       <c r="H52" s="6">
         <f t="shared" si="1"/>
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="I52" s="7">
         <f t="shared" si="2"/>
@@ -3049,29 +2931,29 @@
     </row>
     <row r="53" ht="21.75" customHeight="1">
       <c r="A53" s="9" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="B53" s="10" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="C53" s="10" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="D53" s="9" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="E53" s="11" t="s">
         <v>14</v>
       </c>
       <c r="F53" s="9">
-        <v>45.0</v>
+        <v>25.0</v>
       </c>
       <c r="G53" s="5">
         <v>0.0</v>
       </c>
       <c r="H53" s="12">
         <f t="shared" si="1"/>
-        <v>45</v>
+        <v>25</v>
       </c>
       <c r="I53" s="13">
         <f t="shared" si="2"/>
@@ -3082,76 +2964,8 @@
         <v>À FAIRE</v>
       </c>
     </row>
-    <row r="54" ht="21.75" customHeight="1">
-      <c r="A54" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="B54" s="3" t="s">
-        <v>131</v>
-      </c>
-      <c r="C54" s="3" t="s">
-        <v>132</v>
-      </c>
-      <c r="D54" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="E54" s="17" t="s">
-        <v>25</v>
-      </c>
-      <c r="F54" s="2">
-        <v>30.0</v>
-      </c>
-      <c r="G54" s="5">
-        <v>0.0</v>
-      </c>
-      <c r="H54" s="6">
-        <f t="shared" si="1"/>
-        <v>30</v>
-      </c>
-      <c r="I54" s="7">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="J54" s="8" t="str">
-        <f t="shared" si="3"/>
-        <v>À FAIRE</v>
-      </c>
-    </row>
-    <row r="55" ht="21.75" customHeight="1">
-      <c r="A55" s="9" t="s">
-        <v>126</v>
-      </c>
-      <c r="B55" s="10" t="s">
-        <v>134</v>
-      </c>
-      <c r="C55" s="10" t="s">
-        <v>135</v>
-      </c>
-      <c r="D55" s="9" t="s">
-        <v>133</v>
-      </c>
-      <c r="E55" s="18" t="s">
-        <v>25</v>
-      </c>
-      <c r="F55" s="9">
-        <v>30.0</v>
-      </c>
-      <c r="G55" s="5">
-        <v>0.0</v>
-      </c>
-      <c r="H55" s="12">
-        <f t="shared" si="1"/>
-        <v>30</v>
-      </c>
-      <c r="I55" s="13">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="J55" s="14" t="str">
-        <f t="shared" si="3"/>
-        <v>À FAIRE</v>
-      </c>
-    </row>
+    <row r="54" ht="15.75" customHeight="1"/>
+    <row r="55" ht="15.75" customHeight="1"/>
     <row r="56" ht="15.75" customHeight="1"/>
     <row r="57" ht="15.75" customHeight="1"/>
     <row r="58" ht="15.75" customHeight="1"/>
@@ -4098,17 +3912,17 @@
     <row r="999" ht="15.75" customHeight="1"/>
     <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
-  <conditionalFormatting sqref="J2:J55">
+  <conditionalFormatting sqref="J2:J53">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>"OK"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J2:J55">
+  <conditionalFormatting sqref="J2:J53">
     <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
       <formula>"EN COURS"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J2:J55">
+  <conditionalFormatting sqref="J2:J53">
     <cfRule type="cellIs" dxfId="2" priority="3" operator="equal">
       <formula>"À FAIRE"</formula>
     </cfRule>
@@ -4138,7 +3952,7 @@
   <sheetData>
     <row r="1" ht="30.0" customHeight="1">
       <c r="A1" s="19" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B1" s="20"/>
       <c r="C1" s="20"/>
@@ -4148,53 +3962,53 @@
     </row>
     <row r="2" ht="30.0" customHeight="1">
       <c r="A2" s="22" t="s">
+        <v>135</v>
+      </c>
+      <c r="B2" s="22" t="s">
+        <v>136</v>
+      </c>
+      <c r="C2" s="22" t="s">
         <v>137</v>
       </c>
-      <c r="B2" s="22" t="s">
+      <c r="D2" s="22" t="s">
         <v>138</v>
       </c>
-      <c r="C2" s="22" t="s">
+      <c r="E2" s="22" t="s">
         <v>139</v>
       </c>
-      <c r="D2" s="22" t="s">
+      <c r="F2" s="22" t="s">
         <v>140</v>
-      </c>
-      <c r="E2" s="22" t="s">
-        <v>141</v>
-      </c>
-      <c r="F2" s="22" t="s">
-        <v>142</v>
       </c>
     </row>
     <row r="3" ht="21.75" customHeight="1">
       <c r="A3" s="23">
-        <f>SUM('📋 TODO'!F2:F55)</f>
-        <v>2865</v>
+        <f>SUM(' TODO'!F2:F53)</f>
+        <v>2680</v>
       </c>
       <c r="B3" s="24">
-        <f>SUM('📋 TODO'!G2:G55)</f>
+        <f>SUM(' TODO'!G2:G53)</f>
         <v>0</v>
       </c>
       <c r="C3" s="25">
-        <f>SUM('📋 TODO'!H2:H55)</f>
-        <v>2865</v>
+        <f>SUM(' TODO'!H2:H53)</f>
+        <v>2680</v>
       </c>
       <c r="D3" s="26">
         <f>IFERROR(C3/B3,0)</f>
         <v>0</v>
       </c>
       <c r="E3" s="27">
-        <f>COUNTA('📋 TODO'!A2:A55)</f>
-        <v>54</v>
+        <f>COUNTA(' TODO'!A2:A53)</f>
+        <v>52</v>
       </c>
       <c r="F3" s="24">
-        <f>COUNTIF('📋 TODO'!J2:J55,"OK")</f>
+        <f>COUNTIF(' TODO'!J2:J53,"OK")</f>
         <v>0</v>
       </c>
     </row>
     <row r="5" ht="25.5" customHeight="1">
       <c r="A5" s="28" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="B5" s="20"/>
       <c r="C5" s="20"/>
@@ -4205,10 +4019,10 @@
     </row>
     <row r="6" ht="27.75" customHeight="1">
       <c r="A6" s="22" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B6" s="22" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="C6" s="22" t="s">
         <v>5</v>
@@ -4217,113 +4031,113 @@
         <v>6</v>
       </c>
       <c r="E6" s="22" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="F6" s="22" t="s">
         <v>8</v>
       </c>
       <c r="G6" s="22" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
     </row>
     <row r="7" ht="21.75" customHeight="1">
       <c r="A7" s="29" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="B7" s="30">
-        <f>COUNTIF('📋 TODO'!E2:E55,"Steeven")</f>
-        <v>25</v>
+        <f>COUNTIF(' TODO'!E2:E53,"Steeven")</f>
+        <v>20</v>
       </c>
       <c r="C7" s="30">
-        <f>SUMIF('📋 TODO'!E2:E55,"Steeven",'📋 TODO'!F2:F55)</f>
-        <v>1140</v>
+        <f>SUMIF(' TODO'!E2:E53,"Steeven",' TODO'!F2:F53)</f>
+        <v>950</v>
       </c>
       <c r="D7" s="30">
-        <f>SUMIF('📋 TODO'!E2:E55,"Steeven",'📋 TODO'!G2:G55)</f>
+        <f>SUMIF(' TODO'!E2:E53,"Steeven",' TODO'!G2:G53)</f>
         <v>0</v>
       </c>
       <c r="E7" s="30">
-        <f>SUMIF('📋 TODO'!E2:E55,"Steeven",'📋 TODO'!H2:H55)</f>
-        <v>1140</v>
+        <f>SUMIF(' TODO'!E2:E53,"Steeven",' TODO'!H2:H53)</f>
+        <v>950</v>
       </c>
       <c r="F7" s="31">
         <f t="shared" ref="F7:F10" si="1">IFERROR(D7/C7,0)</f>
         <v>0</v>
       </c>
       <c r="G7" s="30">
-        <f>SUMPRODUCT(('📋 TODO'!E2:E55="Steeven")*('📋 TODO'!J2:J55="OK"))</f>
+        <f>SUMPRODUCT((' TODO'!E2:E53="Steeven")*(' TODO'!J2:J53="OK"))</f>
         <v>0</v>
       </c>
     </row>
     <row r="8" ht="21.75" customHeight="1">
       <c r="A8" s="32" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="B8" s="33">
-        <f>COUNTIF('📋 TODO'!E2:E55,"Mihaja")</f>
-        <v>14</v>
+        <f>COUNTIF(' TODO'!E2:E53,"Mihaja")</f>
+        <v>17</v>
       </c>
       <c r="C8" s="33">
-        <f>SUMIF('📋 TODO'!E2:E55,"Mihaja",'📋 TODO'!F2:F55)</f>
-        <v>870</v>
+        <f>SUMIF(' TODO'!E2:E53,"Mihaja",' TODO'!F2:F53)</f>
+        <v>845</v>
       </c>
       <c r="D8" s="33">
-        <f>SUMIF('📋 TODO'!E2:E55,"Mihaja",'📋 TODO'!G2:G55)</f>
+        <f>SUMIF(' TODO'!E2:E53,"Mihaja",' TODO'!G2:G53)</f>
         <v>0</v>
       </c>
       <c r="E8" s="33">
-        <f>SUMIF('📋 TODO'!E2:E55,"Mihaja",'📋 TODO'!H2:H55)</f>
-        <v>870</v>
+        <f>SUMIF(' TODO'!E2:E53,"Mihaja",' TODO'!H2:H53)</f>
+        <v>845</v>
       </c>
       <c r="F8" s="34">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="G8" s="33">
-        <f>SUMPRODUCT(('📋 TODO'!E2:E55="Mihaja")*('📋 TODO'!J2:J55="OK"))</f>
+        <f>SUMPRODUCT((' TODO'!E2:E53="Mihaja")*(' TODO'!J2:J53="OK"))</f>
         <v>0</v>
       </c>
     </row>
     <row r="9" ht="21.75" customHeight="1">
       <c r="A9" s="35" t="s">
-        <v>14</v>
+        <v>35</v>
       </c>
       <c r="B9" s="30">
-        <f>COUNTIF('📋 TODO'!E2:E55,"Aina")</f>
+        <f>COUNTIF(' TODO'!E2:E53,"Aina")</f>
         <v>15</v>
       </c>
       <c r="C9" s="30">
-        <f>SUMIF('📋 TODO'!E2:E55,"Aina",'📋 TODO'!F2:F55)</f>
-        <v>855</v>
+        <f>SUMIF(' TODO'!E2:E53,"Aina",' TODO'!F2:F53)</f>
+        <v>885</v>
       </c>
       <c r="D9" s="30">
-        <f>SUMIF('📋 TODO'!E2:E55,"Aina",'📋 TODO'!G2:G55)</f>
+        <f>SUMIF(' TODO'!E2:E53,"Aina",' TODO'!G2:G53)</f>
         <v>0</v>
       </c>
       <c r="E9" s="30">
-        <f>SUMIF('📋 TODO'!E2:E55,"Aina",'📋 TODO'!H2:H55)</f>
-        <v>855</v>
+        <f>SUMIF(' TODO'!E2:E53,"Aina",' TODO'!H2:H53)</f>
+        <v>885</v>
       </c>
       <c r="F9" s="36">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="G9" s="30">
-        <f>SUMPRODUCT(('📋 TODO'!E2:E55="Aina")*('📋 TODO'!J2:J55="OK"))</f>
+        <f>SUMPRODUCT((' TODO'!E2:E53="Aina")*(' TODO'!J2:J53="OK"))</f>
         <v>0</v>
       </c>
     </row>
     <row r="10" ht="21.75" customHeight="1">
       <c r="A10" s="37" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="B10" s="38">
         <f t="shared" ref="B10:E10" si="2">SUM(B7:B9)</f>
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C10" s="38">
         <f t="shared" si="2"/>
-        <v>2865</v>
+        <v>2680</v>
       </c>
       <c r="D10" s="38">
         <f t="shared" si="2"/>
@@ -4331,7 +4145,7 @@
       </c>
       <c r="E10" s="38">
         <f t="shared" si="2"/>
-        <v>2865</v>
+        <v>2680</v>
       </c>
       <c r="F10" s="39">
         <f t="shared" si="1"/>
@@ -4342,388 +4156,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" ht="25.5" customHeight="1">
-      <c r="A12" s="28" t="s">
-        <v>148</v>
-      </c>
-      <c r="B12" s="20"/>
-      <c r="C12" s="20"/>
-      <c r="D12" s="20"/>
-      <c r="E12" s="20"/>
-      <c r="F12" s="20"/>
-      <c r="G12" s="21"/>
-    </row>
-    <row r="13" ht="27.75" customHeight="1">
-      <c r="A13" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B13" s="22" t="s">
-        <v>141</v>
-      </c>
-      <c r="C13" s="22" t="s">
-        <v>5</v>
-      </c>
-      <c r="D13" s="22" t="s">
-        <v>6</v>
-      </c>
-      <c r="E13" s="22" t="s">
-        <v>145</v>
-      </c>
-      <c r="F13" s="22" t="s">
-        <v>8</v>
-      </c>
-      <c r="G13" s="22" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="14" ht="19.5" customHeight="1">
-      <c r="A14" s="40" t="s">
-        <v>13</v>
-      </c>
-      <c r="B14" s="33">
-        <f>COUNTIF('📋 TODO'!D2:D55,"HTML/CSS")</f>
-        <v>17</v>
-      </c>
-      <c r="C14" s="33">
-        <f>SUMIF('📋 TODO'!D2:D55,"HTML/CSS",'📋 TODO'!F2:F55)</f>
-        <v>1020</v>
-      </c>
-      <c r="D14" s="33">
-        <f>SUMIF('📋 TODO'!D2:D55,"HTML/CSS",'📋 TODO'!G2:G55)</f>
-        <v>0</v>
-      </c>
-      <c r="E14" s="33">
-        <f>SUMIF('📋 TODO'!D2:D55,"HTML/CSS",'📋 TODO'!H2:H55)</f>
-        <v>1020</v>
-      </c>
-      <c r="F14" s="41">
-        <f t="shared" ref="F14:F25" si="3">IFERROR(D14/C14,0)</f>
-        <v>0</v>
-      </c>
-      <c r="G14" s="33">
-        <f>SUMPRODUCT(('📋 TODO'!D2:D55="HTML/CSS")*('📋 TODO'!J2:J55="OK"))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" ht="19.5" customHeight="1">
-      <c r="A15" s="42" t="s">
-        <v>24</v>
-      </c>
-      <c r="B15" s="30">
-        <f>COUNTIF('📋 TODO'!D2:D55,"PHP/CodeIgniter")</f>
-        <v>15</v>
-      </c>
-      <c r="C15" s="30">
-        <f>SUMIF('📋 TODO'!D2:D55,"PHP/CodeIgniter",'📋 TODO'!F2:F55)</f>
-        <v>820</v>
-      </c>
-      <c r="D15" s="30">
-        <f>SUMIF('📋 TODO'!D2:D55,"PHP/CodeIgniter",'📋 TODO'!G2:G55)</f>
-        <v>0</v>
-      </c>
-      <c r="E15" s="30">
-        <f>SUMIF('📋 TODO'!D2:D55,"PHP/CodeIgniter",'📋 TODO'!H2:H55)</f>
-        <v>820</v>
-      </c>
-      <c r="F15" s="43">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="G15" s="30">
-        <f>SUMPRODUCT(('📋 TODO'!D2:D55="PHP/CodeIgniter")*('📋 TODO'!J2:J55="OK"))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" ht="19.5" customHeight="1">
-      <c r="A16" s="44" t="s">
-        <v>29</v>
-      </c>
-      <c r="B16" s="33">
-        <f>COUNTIF('📋 TODO'!D2:D55,"SQL")</f>
-        <v>7</v>
-      </c>
-      <c r="C16" s="33">
-        <f>SUMIF('📋 TODO'!D2:D55,"SQL",'📋 TODO'!F2:F55)</f>
-        <v>185</v>
-      </c>
-      <c r="D16" s="33">
-        <f>SUMIF('📋 TODO'!D2:D55,"SQL",'📋 TODO'!G2:G55)</f>
-        <v>0</v>
-      </c>
-      <c r="E16" s="33">
-        <f>SUMIF('📋 TODO'!D2:D55,"SQL",'📋 TODO'!H2:H55)</f>
-        <v>185</v>
-      </c>
-      <c r="F16" s="45">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="G16" s="33">
-        <f>SUMPRODUCT(('📋 TODO'!D2:D55="SQL")*('📋 TODO'!J2:J55="OK"))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" ht="19.5" customHeight="1">
-      <c r="A17" s="46" t="s">
-        <v>16</v>
-      </c>
-      <c r="B17" s="30">
-        <f>COUNTIF('📋 TODO'!D2:D55,"JavaScript")</f>
-        <v>3</v>
-      </c>
-      <c r="C17" s="30">
-        <f>SUMIF('📋 TODO'!D2:D55,"JavaScript",'📋 TODO'!F2:F55)</f>
-        <v>180</v>
-      </c>
-      <c r="D17" s="30">
-        <f>SUMIF('📋 TODO'!D2:D55,"JavaScript",'📋 TODO'!G2:G55)</f>
-        <v>0</v>
-      </c>
-      <c r="E17" s="30">
-        <f>SUMIF('📋 TODO'!D2:D55,"JavaScript",'📋 TODO'!H2:H55)</f>
-        <v>180</v>
-      </c>
-      <c r="F17" s="47">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="G17" s="30">
-        <f>SUMPRODUCT(('📋 TODO'!D2:D55="JavaScript")*('📋 TODO'!J2:J55="OK"))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" ht="19.5" customHeight="1">
-      <c r="A18" s="48" t="s">
-        <v>21</v>
-      </c>
-      <c r="B18" s="33">
-        <f>COUNTIF('📋 TODO'!D2:D55,"JavaScript/AJAX")</f>
-        <v>1</v>
-      </c>
-      <c r="C18" s="33">
-        <f>SUMIF('📋 TODO'!D2:D55,"JavaScript/AJAX",'📋 TODO'!F2:F55)</f>
-        <v>60</v>
-      </c>
-      <c r="D18" s="33">
-        <f>SUMIF('📋 TODO'!D2:D55,"JavaScript/AJAX",'📋 TODO'!G2:G55)</f>
-        <v>0</v>
-      </c>
-      <c r="E18" s="33">
-        <f>SUMIF('📋 TODO'!D2:D55,"JavaScript/AJAX",'📋 TODO'!H2:H55)</f>
-        <v>60</v>
-      </c>
-      <c r="F18" s="49">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="G18" s="33">
-        <f>SUMPRODUCT(('📋 TODO'!D2:D55="JavaScript/AJAX")*('📋 TODO'!J2:J55="OK"))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" ht="19.5" customHeight="1">
-      <c r="A19" s="50" t="s">
-        <v>41</v>
-      </c>
-      <c r="B19" s="30">
-        <f>COUNTIF('📋 TODO'!D2:D55,"PHP/AJAX")</f>
-        <v>2</v>
-      </c>
-      <c r="C19" s="30">
-        <f>SUMIF('📋 TODO'!D2:D55,"PHP/AJAX",'📋 TODO'!F2:F55)</f>
-        <v>135</v>
-      </c>
-      <c r="D19" s="30">
-        <f>SUMIF('📋 TODO'!D2:D55,"PHP/AJAX",'📋 TODO'!G2:G55)</f>
-        <v>0</v>
-      </c>
-      <c r="E19" s="30">
-        <f>SUMIF('📋 TODO'!D2:D55,"PHP/AJAX",'📋 TODO'!H2:H55)</f>
-        <v>135</v>
-      </c>
-      <c r="F19" s="51">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="G19" s="30">
-        <f>SUMPRODUCT(('📋 TODO'!D2:D55="PHP/AJAX")*('📋 TODO'!J2:J55="OK"))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" ht="19.5" customHeight="1">
-      <c r="A20" s="52" t="s">
-        <v>85</v>
-      </c>
-      <c r="B20" s="33">
-        <f>COUNTIF('📋 TODO'!D2:D55,"PHP/SQL")</f>
-        <v>1</v>
-      </c>
-      <c r="C20" s="33">
-        <f>SUMIF('📋 TODO'!D2:D55,"PHP/SQL",'📋 TODO'!F2:F55)</f>
-        <v>60</v>
-      </c>
-      <c r="D20" s="33">
-        <f>SUMIF('📋 TODO'!D2:D55,"PHP/SQL",'📋 TODO'!G2:G55)</f>
-        <v>0</v>
-      </c>
-      <c r="E20" s="33">
-        <f>SUMIF('📋 TODO'!D2:D55,"PHP/SQL",'📋 TODO'!H2:H55)</f>
-        <v>60</v>
-      </c>
-      <c r="F20" s="53">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="G20" s="33">
-        <f>SUMPRODUCT(('📋 TODO'!D2:D55="PHP/SQL")*('📋 TODO'!J2:J55="OK"))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" ht="19.5" customHeight="1">
-      <c r="A21" s="42" t="s">
-        <v>58</v>
-      </c>
-      <c r="B21" s="30">
-        <f>COUNTIF('📋 TODO'!D2:D55,"PHP")</f>
-        <v>2</v>
-      </c>
-      <c r="C21" s="30">
-        <f>SUMIF('📋 TODO'!D2:D55,"PHP",'📋 TODO'!F2:F55)</f>
-        <v>135</v>
-      </c>
-      <c r="D21" s="30">
-        <f>SUMIF('📋 TODO'!D2:D55,"PHP",'📋 TODO'!G2:G55)</f>
-        <v>0</v>
-      </c>
-      <c r="E21" s="30">
-        <f>SUMIF('📋 TODO'!D2:D55,"PHP",'📋 TODO'!H2:H55)</f>
-        <v>135</v>
-      </c>
-      <c r="F21" s="43">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="G21" s="30">
-        <f>SUMPRODUCT(('📋 TODO'!D2:D55="PHP")*('📋 TODO'!J2:J55="OK"))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" ht="19.5" customHeight="1">
-      <c r="A22" s="54" t="s">
-        <v>54</v>
-      </c>
-      <c r="B22" s="33">
-        <f>COUNTIF('📋 TODO'!D2:D55,"PHP/HTML")</f>
-        <v>1</v>
-      </c>
-      <c r="C22" s="33">
-        <f>SUMIF('📋 TODO'!D2:D55,"PHP/HTML",'📋 TODO'!F2:F55)</f>
-        <v>45</v>
-      </c>
-      <c r="D22" s="33">
-        <f>SUMIF('📋 TODO'!D2:D55,"PHP/HTML",'📋 TODO'!G2:G55)</f>
-        <v>0</v>
-      </c>
-      <c r="E22" s="33">
-        <f>SUMIF('📋 TODO'!D2:D55,"PHP/HTML",'📋 TODO'!H2:H55)</f>
-        <v>45</v>
-      </c>
-      <c r="F22" s="55">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="G22" s="33">
-        <f>SUMPRODUCT(('📋 TODO'!D2:D55="PHP/HTML")*('📋 TODO'!J2:J55="OK"))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" ht="19.5" customHeight="1">
-      <c r="A23" s="56" t="s">
-        <v>112</v>
-      </c>
-      <c r="B23" s="30">
-        <f>COUNTIF('📋 TODO'!D2:D55,"HTML/CSS/PHP")</f>
-        <v>1</v>
-      </c>
-      <c r="C23" s="30">
-        <f>SUMIF('📋 TODO'!D2:D55,"HTML/CSS/PHP",'📋 TODO'!F2:F55)</f>
-        <v>60</v>
-      </c>
-      <c r="D23" s="30">
-        <f>SUMIF('📋 TODO'!D2:D55,"HTML/CSS/PHP",'📋 TODO'!G2:G55)</f>
-        <v>0</v>
-      </c>
-      <c r="E23" s="30">
-        <f>SUMIF('📋 TODO'!D2:D55,"HTML/CSS/PHP",'📋 TODO'!H2:H55)</f>
-        <v>60</v>
-      </c>
-      <c r="F23" s="57">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="G23" s="30">
-        <f>SUMPRODUCT(('📋 TODO'!D2:D55="HTML/CSS/PHP")*('📋 TODO'!J2:J55="OK"))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" ht="19.5" customHeight="1">
-      <c r="A24" s="58" t="s">
-        <v>129</v>
-      </c>
-      <c r="B24" s="33">
-        <f>COUNTIF('📋 TODO'!D2:D55,"Tests")</f>
-        <v>2</v>
-      </c>
-      <c r="C24" s="33">
-        <f>SUMIF('📋 TODO'!D2:D55,"Tests",'📋 TODO'!F2:F55)</f>
-        <v>105</v>
-      </c>
-      <c r="D24" s="33">
-        <f>SUMIF('📋 TODO'!D2:D55,"Tests",'📋 TODO'!G2:G55)</f>
-        <v>0</v>
-      </c>
-      <c r="E24" s="33">
-        <f>SUMIF('📋 TODO'!D2:D55,"Tests",'📋 TODO'!H2:H55)</f>
-        <v>105</v>
-      </c>
-      <c r="F24" s="59">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="G24" s="33">
-        <f>SUMPRODUCT(('📋 TODO'!D2:D55="Tests")*('📋 TODO'!J2:J55="OK"))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" ht="19.5" customHeight="1">
-      <c r="A25" s="60" t="s">
-        <v>133</v>
-      </c>
-      <c r="B25" s="30">
-        <f>COUNTIF('📋 TODO'!D2:D55,"Général")</f>
-        <v>2</v>
-      </c>
-      <c r="C25" s="30">
-        <f>SUMIF('📋 TODO'!D2:D55,"Général",'📋 TODO'!F2:F55)</f>
-        <v>60</v>
-      </c>
-      <c r="D25" s="30">
-        <f>SUMIF('📋 TODO'!D2:D55,"Général",'📋 TODO'!G2:G55)</f>
-        <v>0</v>
-      </c>
-      <c r="E25" s="30">
-        <f>SUMIF('📋 TODO'!D2:D55,"Général",'📋 TODO'!H2:H55)</f>
-        <v>60</v>
-      </c>
-      <c r="F25" s="61">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="G25" s="30">
-        <f>SUMPRODUCT(('📋 TODO'!D2:D55="Général")*('📋 TODO'!J2:J55="OK"))</f>
-        <v>0</v>
-      </c>
-    </row>
+    <row r="21" ht="15.75" customHeight="1"/>
+    <row r="22" ht="15.75" customHeight="1"/>
+    <row r="23" ht="15.75" customHeight="1"/>
+    <row r="24" ht="15.75" customHeight="1"/>
+    <row r="25" ht="15.75" customHeight="1"/>
     <row r="26" ht="15.75" customHeight="1"/>
     <row r="27" ht="15.75" customHeight="1"/>
     <row r="28" ht="15.75" customHeight="1"/>
@@ -5700,10 +5137,9 @@
     <row r="999" ht="15.75" customHeight="1"/>
     <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="2">
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A5:G5"/>
-    <mergeCell ref="A12:G12"/>
   </mergeCells>
   <printOptions/>
   <pageMargins bottom="1.0" footer="0.0" header="0.0" left="0.75" right="0.75" top="1.0"/>
@@ -5726,7 +5162,7 @@
   <sheetData>
     <row r="1" ht="27.75" customHeight="1">
       <c r="A1" s="28" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="B1" s="20"/>
       <c r="C1" s="20"/>
@@ -5735,403 +5171,403 @@
     </row>
     <row r="2" ht="27.75" customHeight="1">
       <c r="A2" s="22" t="s">
+        <v>147</v>
+      </c>
+      <c r="B2" s="22" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" s="22" t="s">
+        <v>30</v>
+      </c>
+      <c r="D2" s="22" t="s">
+        <v>35</v>
+      </c>
+      <c r="E2" s="22" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="3" ht="19.5" customHeight="1">
+      <c r="A3" s="40" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="41">
+        <f>SUMPRODUCT((' TODO'!A2:A53="INSCRIPTION")*(' TODO'!E2:E53="Steeven")*(' TODO'!F2:F53))</f>
+        <v>310</v>
+      </c>
+      <c r="C3" s="42">
+        <f>SUMPRODUCT((' TODO'!A2:A53="INSCRIPTION")*(' TODO'!E2:E53="Mihaja")*(' TODO'!F2:F53))</f>
+        <v>0</v>
+      </c>
+      <c r="D3" s="43">
+        <f>SUMPRODUCT((' TODO'!A2:A53="INSCRIPTION")*(' TODO'!E2:E53="Aina")*(' TODO'!F2:F53))</f>
+        <v>0</v>
+      </c>
+      <c r="E3" s="44">
+        <f t="shared" ref="E3:E19" si="1">SUM(B3:D3)</f>
+        <v>310</v>
+      </c>
+    </row>
+    <row r="4" ht="19.5" customHeight="1">
+      <c r="A4" s="45" t="s">
+        <v>27</v>
+      </c>
+      <c r="B4" s="46">
+        <f>SUMPRODUCT((' TODO'!A2:A53="LOGIN")*(' TODO'!E2:E53="Steeven")*(' TODO'!F2:F53))</f>
+        <v>0</v>
+      </c>
+      <c r="C4" s="47">
+        <f>SUMPRODUCT((' TODO'!A2:A53="LOGIN")*(' TODO'!E2:E53="Mihaja")*(' TODO'!F2:F53))</f>
+        <v>110</v>
+      </c>
+      <c r="D4" s="48">
+        <f>SUMPRODUCT((' TODO'!A2:A53="LOGIN")*(' TODO'!E2:E53="Aina")*(' TODO'!F2:F53))</f>
+        <v>0</v>
+      </c>
+      <c r="E4" s="27">
+        <f t="shared" si="1"/>
+        <v>110</v>
+      </c>
+    </row>
+    <row r="5" ht="19.5" customHeight="1">
+      <c r="A5" s="40" t="s">
+        <v>32</v>
+      </c>
+      <c r="B5" s="41">
+        <f>SUMPRODUCT((' TODO'!A2:A53="PROFIL")*(' TODO'!E2:E53="Steeven")*(' TODO'!F2:F53))</f>
+        <v>0</v>
+      </c>
+      <c r="C5" s="42">
+        <f>SUMPRODUCT((' TODO'!A2:A53="PROFIL")*(' TODO'!E2:E53="Mihaja")*(' TODO'!F2:F53))</f>
+        <v>0</v>
+      </c>
+      <c r="D5" s="43">
+        <f>SUMPRODUCT((' TODO'!A2:A53="PROFIL")*(' TODO'!E2:E53="Aina")*(' TODO'!F2:F53))</f>
+        <v>120</v>
+      </c>
+      <c r="E5" s="44">
+        <f t="shared" si="1"/>
+        <v>120</v>
+      </c>
+    </row>
+    <row r="6" ht="19.5" customHeight="1">
+      <c r="A6" s="45" t="s">
+        <v>39</v>
+      </c>
+      <c r="B6" s="46">
+        <f>SUMPRODUCT((' TODO'!A2:A53="OBJECTIF")*(' TODO'!E2:E53="Steeven")*(' TODO'!F2:F53))</f>
+        <v>0</v>
+      </c>
+      <c r="C6" s="47">
+        <f>SUMPRODUCT((' TODO'!A2:A53="OBJECTIF")*(' TODO'!E2:E53="Mihaja")*(' TODO'!F2:F53))</f>
+        <v>90</v>
+      </c>
+      <c r="D6" s="48">
+        <f>SUMPRODUCT((' TODO'!A2:A53="OBJECTIF")*(' TODO'!E2:E53="Aina")*(' TODO'!F2:F53))</f>
+        <v>0</v>
+      </c>
+      <c r="E6" s="27">
+        <f t="shared" si="1"/>
+        <v>90</v>
+      </c>
+    </row>
+    <row r="7" ht="19.5" customHeight="1">
+      <c r="A7" s="40" t="s">
+        <v>44</v>
+      </c>
+      <c r="B7" s="41">
+        <f>SUMPRODUCT((' TODO'!A2:A53="SUGGESTION")*(' TODO'!E2:E53="Steeven")*(' TODO'!F2:F53))</f>
+        <v>55</v>
+      </c>
+      <c r="C7" s="42">
+        <f>SUMPRODUCT((' TODO'!A2:A53="SUGGESTION")*(' TODO'!E2:E53="Mihaja")*(' TODO'!F2:F53))</f>
+        <v>0</v>
+      </c>
+      <c r="D7" s="43">
+        <f>SUMPRODUCT((' TODO'!A2:A53="SUGGESTION")*(' TODO'!E2:E53="Aina")*(' TODO'!F2:F53))</f>
+        <v>240</v>
+      </c>
+      <c r="E7" s="44">
+        <f t="shared" si="1"/>
+        <v>295</v>
+      </c>
+    </row>
+    <row r="8" ht="19.5" customHeight="1">
+      <c r="A8" s="45" t="s">
+        <v>51</v>
+      </c>
+      <c r="B8" s="46">
+        <f>SUMPRODUCT((' TODO'!A2:A53="EXPORT PDF")*(' TODO'!E2:E53="Steeven")*(' TODO'!F2:F53))</f>
+        <v>0</v>
+      </c>
+      <c r="C8" s="47">
+        <f>SUMPRODUCT((' TODO'!A2:A53="EXPORT PDF")*(' TODO'!E2:E53="Mihaja")*(' TODO'!F2:F53))</f>
+        <v>135</v>
+      </c>
+      <c r="D8" s="48">
+        <f>SUMPRODUCT((' TODO'!A2:A53="EXPORT PDF")*(' TODO'!E2:E53="Aina")*(' TODO'!F2:F53))</f>
+        <v>0</v>
+      </c>
+      <c r="E8" s="27">
+        <f t="shared" si="1"/>
+        <v>135</v>
+      </c>
+    </row>
+    <row r="9" ht="19.5" customHeight="1">
+      <c r="A9" s="40" t="s">
+        <v>56</v>
+      </c>
+      <c r="B9" s="41">
+        <f>SUMPRODUCT((' TODO'!A2:A53="PORTE MONNAIE")*(' TODO'!E2:E53="Steeven")*(' TODO'!F2:F53))</f>
+        <v>125</v>
+      </c>
+      <c r="C9" s="42">
+        <f>SUMPRODUCT((' TODO'!A2:A53="PORTE MONNAIE")*(' TODO'!E2:E53="Mihaja")*(' TODO'!F2:F53))</f>
+        <v>0</v>
+      </c>
+      <c r="D9" s="43">
+        <f>SUMPRODUCT((' TODO'!A2:A53="PORTE MONNAIE")*(' TODO'!E2:E53="Aina")*(' TODO'!F2:F53))</f>
+        <v>0</v>
+      </c>
+      <c r="E9" s="44">
+        <f t="shared" si="1"/>
+        <v>125</v>
+      </c>
+    </row>
+    <row r="10" ht="19.5" customHeight="1">
+      <c r="A10" s="45" t="s">
+        <v>63</v>
+      </c>
+      <c r="B10" s="46">
+        <f>SUMPRODUCT((' TODO'!A2:A53="OPTION GOLD")*(' TODO'!E2:E53="Steeven")*(' TODO'!F2:F53))</f>
+        <v>30</v>
+      </c>
+      <c r="C10" s="47">
+        <f>SUMPRODUCT((' TODO'!A2:A53="OPTION GOLD")*(' TODO'!E2:E53="Mihaja")*(' TODO'!F2:F53))</f>
+        <v>105</v>
+      </c>
+      <c r="D10" s="48">
+        <f>SUMPRODUCT((' TODO'!A2:A53="OPTION GOLD")*(' TODO'!E2:E53="Aina")*(' TODO'!F2:F53))</f>
+        <v>0</v>
+      </c>
+      <c r="E10" s="27">
+        <f t="shared" si="1"/>
+        <v>135</v>
+      </c>
+    </row>
+    <row r="11" ht="19.5" customHeight="1">
+      <c r="A11" s="40" t="s">
+        <v>69</v>
+      </c>
+      <c r="B11" s="41">
+        <f>SUMPRODUCT((' TODO'!A2:A53="NAVIGATION")*(' TODO'!E2:E53="Steeven")*(' TODO'!F2:F53))</f>
+        <v>0</v>
+      </c>
+      <c r="C11" s="42">
+        <f>SUMPRODUCT((' TODO'!A2:A53="NAVIGATION")*(' TODO'!E2:E53="Mihaja")*(' TODO'!F2:F53))</f>
+        <v>0</v>
+      </c>
+      <c r="D11" s="43">
+        <f>SUMPRODUCT((' TODO'!A2:A53="NAVIGATION")*(' TODO'!E2:E53="Aina")*(' TODO'!F2:F53))</f>
+        <v>105</v>
+      </c>
+      <c r="E11" s="44">
+        <f t="shared" si="1"/>
+        <v>105</v>
+      </c>
+    </row>
+    <row r="12" ht="19.5" customHeight="1">
+      <c r="A12" s="45" t="s">
+        <v>74</v>
+      </c>
+      <c r="B12" s="46">
+        <f>SUMPRODUCT((' TODO'!A2:A53="BO LOGIN")*(' TODO'!E2:E53="Steeven")*(' TODO'!F2:F53))</f>
+        <v>0</v>
+      </c>
+      <c r="C12" s="47">
+        <f>SUMPRODUCT((' TODO'!A2:A53="BO LOGIN")*(' TODO'!E2:E53="Mihaja")*(' TODO'!F2:F53))</f>
+        <v>80</v>
+      </c>
+      <c r="D12" s="48">
+        <f>SUMPRODUCT((' TODO'!A2:A53="BO LOGIN")*(' TODO'!E2:E53="Aina")*(' TODO'!F2:F53))</f>
+        <v>0</v>
+      </c>
+      <c r="E12" s="27">
+        <f t="shared" si="1"/>
+        <v>80</v>
+      </c>
+    </row>
+    <row r="13" ht="19.5" customHeight="1">
+      <c r="A13" s="40" t="s">
+        <v>79</v>
+      </c>
+      <c r="B13" s="41">
+        <f>SUMPRODUCT((' TODO'!A2:A53="BO DASHBOARD")*(' TODO'!E2:E53="Steeven")*(' TODO'!F2:F53))</f>
+        <v>75</v>
+      </c>
+      <c r="C13" s="42">
+        <f>SUMPRODUCT((' TODO'!A2:A53="BO DASHBOARD")*(' TODO'!E2:E53="Mihaja")*(' TODO'!F2:F53))</f>
+        <v>60</v>
+      </c>
+      <c r="D13" s="43">
+        <f>SUMPRODUCT((' TODO'!A2:A53="BO DASHBOARD")*(' TODO'!E2:E53="Aina")*(' TODO'!F2:F53))</f>
+        <v>135</v>
+      </c>
+      <c r="E13" s="44">
+        <f t="shared" si="1"/>
+        <v>270</v>
+      </c>
+    </row>
+    <row r="14" ht="19.5" customHeight="1">
+      <c r="A14" s="45" t="s">
+        <v>87</v>
+      </c>
+      <c r="B14" s="46">
+        <f>SUMPRODUCT((' TODO'!A2:A53="BO RÉGIMES")*(' TODO'!E2:E53="Steeven")*(' TODO'!F2:F53))</f>
+        <v>105</v>
+      </c>
+      <c r="C14" s="47">
+        <f>SUMPRODUCT((' TODO'!A2:A53="BO RÉGIMES")*(' TODO'!E2:E53="Mihaja")*(' TODO'!F2:F53))</f>
+        <v>65</v>
+      </c>
+      <c r="D14" s="48">
+        <f>SUMPRODUCT((' TODO'!A2:A53="BO RÉGIMES")*(' TODO'!E2:E53="Aina")*(' TODO'!F2:F53))</f>
+        <v>55</v>
+      </c>
+      <c r="E14" s="27">
+        <f t="shared" si="1"/>
+        <v>225</v>
+      </c>
+    </row>
+    <row r="15" ht="19.5" customHeight="1">
+      <c r="A15" s="40" t="s">
+        <v>96</v>
+      </c>
+      <c r="B15" s="41">
+        <f>SUMPRODUCT((' TODO'!A2:A53="BO ACTIVITÉS")*(' TODO'!E2:E53="Steeven")*(' TODO'!F2:F53))</f>
+        <v>0</v>
+      </c>
+      <c r="C15" s="42">
+        <f>SUMPRODUCT((' TODO'!A2:A53="BO ACTIVITÉS")*(' TODO'!E2:E53="Mihaja")*(' TODO'!F2:F53))</f>
+        <v>75</v>
+      </c>
+      <c r="D15" s="43">
+        <f>SUMPRODUCT((' TODO'!A2:A53="BO ACTIVITÉS")*(' TODO'!E2:E53="Aina")*(' TODO'!F2:F53))</f>
+        <v>90</v>
+      </c>
+      <c r="E15" s="44">
+        <f t="shared" si="1"/>
+        <v>165</v>
+      </c>
+    </row>
+    <row r="16" ht="19.5" customHeight="1">
+      <c r="A16" s="45" t="s">
+        <v>105</v>
+      </c>
+      <c r="B16" s="46">
+        <f>SUMPRODUCT((' TODO'!A2:A53="BO CODES")*(' TODO'!E2:E53="Steeven")*(' TODO'!F2:F53))</f>
         <v>150</v>
       </c>
-      <c r="B2" s="22" t="s">
-        <v>25</v>
-      </c>
-      <c r="C2" s="22" t="s">
-        <v>19</v>
-      </c>
-      <c r="D2" s="22" t="s">
-        <v>14</v>
-      </c>
-      <c r="E2" s="22" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="3" ht="19.5" customHeight="1">
-      <c r="A3" s="62" t="s">
+      <c r="C16" s="47">
+        <f>SUMPRODUCT((' TODO'!A2:A53="BO CODES")*(' TODO'!E2:E53="Mihaja")*(' TODO'!F2:F53))</f>
+        <v>0</v>
+      </c>
+      <c r="D16" s="48">
+        <f>SUMPRODUCT((' TODO'!A2:A53="BO CODES")*(' TODO'!E2:E53="Aina")*(' TODO'!F2:F53))</f>
+        <v>0</v>
+      </c>
+      <c r="E16" s="27">
+        <f t="shared" si="1"/>
+        <v>150</v>
+      </c>
+    </row>
+    <row r="17" ht="19.5" customHeight="1">
+      <c r="A17" s="40" t="s">
+        <v>112</v>
+      </c>
+      <c r="B17" s="41">
+        <f>SUMPRODUCT((' TODO'!A2:A53="BO PARAMÈTRES")*(' TODO'!E2:E53="Steeven")*(' TODO'!F2:F53))</f>
+        <v>0</v>
+      </c>
+      <c r="C17" s="42">
+        <f>SUMPRODUCT((' TODO'!A2:A53="BO PARAMÈTRES")*(' TODO'!E2:E53="Mihaja")*(' TODO'!F2:F53))</f>
         <v>10</v>
       </c>
-      <c r="B3" s="63">
-        <f>SUMPRODUCT(('📋 TODO'!A2:A55="INSCRIPTION")*('📋 TODO'!E2:E55="Steeven")*('📋 TODO'!F2:F55))</f>
-        <v>140</v>
-      </c>
-      <c r="C3" s="64">
-        <f>SUMPRODUCT(('📋 TODO'!A2:A55="INSCRIPTION")*('📋 TODO'!E2:E55="Mihaja")*('📋 TODO'!F2:F55))</f>
-        <v>120</v>
-      </c>
-      <c r="D3" s="65">
-        <f>SUMPRODUCT(('📋 TODO'!A2:A55="INSCRIPTION")*('📋 TODO'!E2:E55="Aina")*('📋 TODO'!F2:F55))</f>
-        <v>135</v>
-      </c>
-      <c r="E3" s="66">
-        <f t="shared" ref="E3:E19" si="1">SUM(B3:D3)</f>
-        <v>395</v>
-      </c>
-    </row>
-    <row r="4" ht="19.5" customHeight="1">
-      <c r="A4" s="67" t="s">
-        <v>30</v>
-      </c>
-      <c r="B4" s="68">
-        <f>SUMPRODUCT(('📋 TODO'!A2:A55="LOGIN")*('📋 TODO'!E2:E55="Steeven")*('📋 TODO'!F2:F55))</f>
+      <c r="D17" s="43">
+        <f>SUMPRODUCT((' TODO'!A2:A53="BO PARAMÈTRES")*(' TODO'!E2:E53="Aina")*(' TODO'!F2:F53))</f>
         <v>90</v>
       </c>
-      <c r="C4" s="69">
-        <f>SUMPRODUCT(('📋 TODO'!A2:A55="LOGIN")*('📋 TODO'!E2:E55="Mihaja")*('📋 TODO'!F2:F55))</f>
-        <v>0</v>
-      </c>
-      <c r="D4" s="70">
-        <f>SUMPRODUCT(('📋 TODO'!A2:A55="LOGIN")*('📋 TODO'!E2:E55="Aina")*('📋 TODO'!F2:F55))</f>
+      <c r="E17" s="44">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="18" ht="19.5" customHeight="1">
+      <c r="A18" s="45" t="s">
+        <v>119</v>
+      </c>
+      <c r="B18" s="46">
+        <f>SUMPRODUCT((' TODO'!A2:A53="BASE DE DONNÉES")*(' TODO'!E2:E53="Steeven")*(' TODO'!F2:F53))</f>
         <v>45</v>
       </c>
-      <c r="E4" s="27">
-        <f t="shared" si="1"/>
-        <v>135</v>
-      </c>
-    </row>
-    <row r="5" ht="19.5" customHeight="1">
-      <c r="A5" s="62" t="s">
-        <v>36</v>
-      </c>
-      <c r="B5" s="63">
-        <f>SUMPRODUCT(('📋 TODO'!A2:A55="PROFIL")*('📋 TODO'!E2:E55="Steeven")*('📋 TODO'!F2:F55))</f>
+      <c r="C18" s="47">
+        <f>SUMPRODUCT((' TODO'!A2:A53="BASE DE DONNÉES")*(' TODO'!E2:E53="Mihaja")*(' TODO'!F2:F53))</f>
+        <v>55</v>
+      </c>
+      <c r="D18" s="48">
+        <f>SUMPRODUCT((' TODO'!A2:A53="BASE DE DONNÉES")*(' TODO'!E2:E53="Aina")*(' TODO'!F2:F53))</f>
+        <v>0</v>
+      </c>
+      <c r="E18" s="27">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="19" ht="19.5" customHeight="1">
+      <c r="A19" s="40" t="s">
+        <v>124</v>
+      </c>
+      <c r="B19" s="41">
+        <f>SUMPRODUCT((' TODO'!A2:A53="TESTS &amp; LIVRAISON")*(' TODO'!E2:E53="Steeven")*(' TODO'!F2:F53))</f>
+        <v>55</v>
+      </c>
+      <c r="C19" s="42">
+        <f>SUMPRODUCT((' TODO'!A2:A53="TESTS &amp; LIVRAISON")*(' TODO'!E2:E53="Mihaja")*(' TODO'!F2:F53))</f>
         <v>60</v>
       </c>
-      <c r="C5" s="64">
-        <f>SUMPRODUCT(('📋 TODO'!A2:A55="PROFIL")*('📋 TODO'!E2:E55="Mihaja")*('📋 TODO'!F2:F55))</f>
-        <v>0</v>
-      </c>
-      <c r="D5" s="65">
-        <f>SUMPRODUCT(('📋 TODO'!A2:A55="PROFIL")*('📋 TODO'!E2:E55="Aina")*('📋 TODO'!F2:F55))</f>
-        <v>60</v>
-      </c>
-      <c r="E5" s="66">
-        <f t="shared" si="1"/>
-        <v>120</v>
-      </c>
-    </row>
-    <row r="6" ht="19.5" customHeight="1">
-      <c r="A6" s="67" t="s">
-        <v>42</v>
-      </c>
-      <c r="B6" s="68">
-        <f>SUMPRODUCT(('📋 TODO'!A2:A55="OBJECTIF")*('📋 TODO'!E2:E55="Steeven")*('📋 TODO'!F2:F55))</f>
-        <v>30</v>
-      </c>
-      <c r="C6" s="69">
-        <f>SUMPRODUCT(('📋 TODO'!A2:A55="OBJECTIF")*('📋 TODO'!E2:E55="Mihaja")*('📋 TODO'!F2:F55))</f>
-        <v>0</v>
-      </c>
-      <c r="D6" s="70">
-        <f>SUMPRODUCT(('📋 TODO'!A2:A55="OBJECTIF")*('📋 TODO'!E2:E55="Aina")*('📋 TODO'!F2:F55))</f>
-        <v>60</v>
-      </c>
-      <c r="E6" s="27">
-        <f t="shared" si="1"/>
-        <v>90</v>
-      </c>
-    </row>
-    <row r="7" ht="19.5" customHeight="1">
-      <c r="A7" s="62" t="s">
-        <v>47</v>
-      </c>
-      <c r="B7" s="63">
-        <f>SUMPRODUCT(('📋 TODO'!A2:A55="SUGGESTION")*('📋 TODO'!E2:E55="Steeven")*('📋 TODO'!F2:F55))</f>
-        <v>180</v>
-      </c>
-      <c r="C7" s="64">
-        <f>SUMPRODUCT(('📋 TODO'!A2:A55="SUGGESTION")*('📋 TODO'!E2:E55="Mihaja")*('📋 TODO'!F2:F55))</f>
-        <v>45</v>
-      </c>
-      <c r="D7" s="65">
-        <f>SUMPRODUCT(('📋 TODO'!A2:A55="SUGGESTION")*('📋 TODO'!E2:E55="Aina")*('📋 TODO'!F2:F55))</f>
-        <v>90</v>
-      </c>
-      <c r="E7" s="66">
-        <f t="shared" si="1"/>
-        <v>315</v>
-      </c>
-    </row>
-    <row r="8" ht="19.5" customHeight="1">
-      <c r="A8" s="67" t="s">
-        <v>55</v>
-      </c>
-      <c r="B8" s="68">
-        <f>SUMPRODUCT(('📋 TODO'!A2:A55="EXPORT PDF")*('📋 TODO'!E2:E55="Steeven")*('📋 TODO'!F2:F55))</f>
-        <v>0</v>
-      </c>
-      <c r="C8" s="69">
-        <f>SUMPRODUCT(('📋 TODO'!A2:A55="EXPORT PDF")*('📋 TODO'!E2:E55="Mihaja")*('📋 TODO'!F2:F55))</f>
-        <v>135</v>
-      </c>
-      <c r="D8" s="70">
-        <f>SUMPRODUCT(('📋 TODO'!A2:A55="EXPORT PDF")*('📋 TODO'!E2:E55="Aina")*('📋 TODO'!F2:F55))</f>
-        <v>0</v>
-      </c>
-      <c r="E8" s="27">
-        <f t="shared" si="1"/>
-        <v>135</v>
-      </c>
-    </row>
-    <row r="9" ht="19.5" customHeight="1">
-      <c r="A9" s="62" t="s">
-        <v>60</v>
-      </c>
-      <c r="B9" s="63">
-        <f>SUMPRODUCT(('📋 TODO'!A2:A55="PORTE MONNAIE")*('📋 TODO'!E2:E55="Steeven")*('📋 TODO'!F2:F55))</f>
-        <v>90</v>
-      </c>
-      <c r="C9" s="64">
-        <f>SUMPRODUCT(('📋 TODO'!A2:A55="PORTE MONNAIE")*('📋 TODO'!E2:E55="Mihaja")*('📋 TODO'!F2:F55))</f>
-        <v>0</v>
-      </c>
-      <c r="D9" s="65">
-        <f>SUMPRODUCT(('📋 TODO'!A2:A55="PORTE MONNAIE")*('📋 TODO'!E2:E55="Aina")*('📋 TODO'!F2:F55))</f>
-        <v>45</v>
-      </c>
-      <c r="E9" s="66">
-        <f t="shared" si="1"/>
-        <v>135</v>
-      </c>
-    </row>
-    <row r="10" ht="19.5" customHeight="1">
-      <c r="A10" s="67" t="s">
-        <v>67</v>
-      </c>
-      <c r="B10" s="68">
-        <f>SUMPRODUCT(('📋 TODO'!A2:A55="OPTION GOLD")*('📋 TODO'!E2:E55="Steeven")*('📋 TODO'!F2:F55))</f>
-        <v>30</v>
-      </c>
-      <c r="C10" s="69">
-        <f>SUMPRODUCT(('📋 TODO'!A2:A55="OPTION GOLD")*('📋 TODO'!E2:E55="Mihaja")*('📋 TODO'!F2:F55))</f>
-        <v>60</v>
-      </c>
-      <c r="D10" s="70">
-        <f>SUMPRODUCT(('📋 TODO'!A2:A55="OPTION GOLD")*('📋 TODO'!E2:E55="Aina")*('📋 TODO'!F2:F55))</f>
-        <v>45</v>
-      </c>
-      <c r="E10" s="27">
-        <f t="shared" si="1"/>
-        <v>135</v>
-      </c>
-    </row>
-    <row r="11" ht="19.5" customHeight="1">
-      <c r="A11" s="62" t="s">
-        <v>73</v>
-      </c>
-      <c r="B11" s="63">
-        <f>SUMPRODUCT(('📋 TODO'!A2:A55="BO LOGIN")*('📋 TODO'!E2:E55="Steeven")*('📋 TODO'!F2:F55))</f>
-        <v>40</v>
-      </c>
-      <c r="C11" s="64">
-        <f>SUMPRODUCT(('📋 TODO'!A2:A55="BO LOGIN")*('📋 TODO'!E2:E55="Mihaja")*('📋 TODO'!F2:F55))</f>
-        <v>0</v>
-      </c>
-      <c r="D11" s="65">
-        <f>SUMPRODUCT(('📋 TODO'!A2:A55="BO LOGIN")*('📋 TODO'!E2:E55="Aina")*('📋 TODO'!F2:F55))</f>
-        <v>30</v>
-      </c>
-      <c r="E11" s="66">
-        <f t="shared" si="1"/>
-        <v>70</v>
-      </c>
-    </row>
-    <row r="12" ht="19.5" customHeight="1">
-      <c r="A12" s="67" t="s">
-        <v>78</v>
-      </c>
-      <c r="B12" s="68">
-        <f>SUMPRODUCT(('📋 TODO'!A2:A55="BO DASHBOARD")*('📋 TODO'!E2:E55="Steeven")*('📋 TODO'!F2:F55))</f>
-        <v>60</v>
-      </c>
-      <c r="C12" s="69">
-        <f>SUMPRODUCT(('📋 TODO'!A2:A55="BO DASHBOARD")*('📋 TODO'!E2:E55="Mihaja")*('📋 TODO'!F2:F55))</f>
-        <v>165</v>
-      </c>
-      <c r="D12" s="70">
-        <f>SUMPRODUCT(('📋 TODO'!A2:A55="BO DASHBOARD")*('📋 TODO'!E2:E55="Aina")*('📋 TODO'!F2:F55))</f>
-        <v>60</v>
-      </c>
-      <c r="E12" s="27">
-        <f t="shared" si="1"/>
-        <v>285</v>
-      </c>
-    </row>
-    <row r="13" ht="19.5" customHeight="1">
-      <c r="A13" s="62" t="s">
-        <v>86</v>
-      </c>
-      <c r="B13" s="63">
-        <f>SUMPRODUCT(('📋 TODO'!A2:A55="BO RÉGIMES")*('📋 TODO'!E2:E55="Steeven")*('📋 TODO'!F2:F55))</f>
-        <v>110</v>
-      </c>
-      <c r="C13" s="64">
-        <f>SUMPRODUCT(('📋 TODO'!A2:A55="BO RÉGIMES")*('📋 TODO'!E2:E55="Mihaja")*('📋 TODO'!F2:F55))</f>
-        <v>75</v>
-      </c>
-      <c r="D13" s="65">
-        <f>SUMPRODUCT(('📋 TODO'!A2:A55="BO RÉGIMES")*('📋 TODO'!E2:E55="Aina")*('📋 TODO'!F2:F55))</f>
-        <v>60</v>
-      </c>
-      <c r="E13" s="66">
-        <f t="shared" si="1"/>
-        <v>245</v>
-      </c>
-    </row>
-    <row r="14" ht="19.5" customHeight="1">
-      <c r="A14" s="67" t="s">
-        <v>95</v>
-      </c>
-      <c r="B14" s="68">
-        <f>SUMPRODUCT(('📋 TODO'!A2:A55="BO ACTIVITÉS")*('📋 TODO'!E2:E55="Steeven")*('📋 TODO'!F2:F55))</f>
-        <v>75</v>
-      </c>
-      <c r="C14" s="69">
-        <f>SUMPRODUCT(('📋 TODO'!A2:A55="BO ACTIVITÉS")*('📋 TODO'!E2:E55="Mihaja")*('📋 TODO'!F2:F55))</f>
-        <v>0</v>
-      </c>
-      <c r="D14" s="70">
-        <f>SUMPRODUCT(('📋 TODO'!A2:A55="BO ACTIVITÉS")*('📋 TODO'!E2:E55="Aina")*('📋 TODO'!F2:F55))</f>
-        <v>60</v>
-      </c>
-      <c r="E14" s="27">
-        <f t="shared" si="1"/>
-        <v>135</v>
-      </c>
-    </row>
-    <row r="15" ht="19.5" customHeight="1">
-      <c r="A15" s="62" t="s">
-        <v>102</v>
-      </c>
-      <c r="B15" s="63">
-        <f>SUMPRODUCT(('📋 TODO'!A2:A55="BO CODES")*('📋 TODO'!E2:E55="Steeven")*('📋 TODO'!F2:F55))</f>
-        <v>75</v>
-      </c>
-      <c r="C15" s="64">
-        <f>SUMPRODUCT(('📋 TODO'!A2:A55="BO CODES")*('📋 TODO'!E2:E55="Mihaja")*('📋 TODO'!F2:F55))</f>
-        <v>90</v>
-      </c>
-      <c r="D15" s="65">
-        <f>SUMPRODUCT(('📋 TODO'!A2:A55="BO CODES")*('📋 TODO'!E2:E55="Aina")*('📋 TODO'!F2:F55))</f>
-        <v>0</v>
-      </c>
-      <c r="E15" s="66">
-        <f t="shared" si="1"/>
-        <v>165</v>
-      </c>
-    </row>
-    <row r="16" ht="19.5" customHeight="1">
-      <c r="A16" s="67" t="s">
-        <v>109</v>
-      </c>
-      <c r="B16" s="68">
-        <f>SUMPRODUCT(('📋 TODO'!A2:A55="BO PARAMÈTRES")*('📋 TODO'!E2:E55="Steeven")*('📋 TODO'!F2:F55))</f>
-        <v>55</v>
-      </c>
-      <c r="C16" s="69">
-        <f>SUMPRODUCT(('📋 TODO'!A2:A55="BO PARAMÈTRES")*('📋 TODO'!E2:E55="Mihaja")*('📋 TODO'!F2:F55))</f>
-        <v>60</v>
-      </c>
-      <c r="D16" s="70">
-        <f>SUMPRODUCT(('📋 TODO'!A2:A55="BO PARAMÈTRES")*('📋 TODO'!E2:E55="Aina")*('📋 TODO'!F2:F55))</f>
-        <v>0</v>
-      </c>
-      <c r="E16" s="27">
-        <f t="shared" si="1"/>
-        <v>115</v>
-      </c>
-    </row>
-    <row r="17" ht="19.5" customHeight="1">
-      <c r="A17" s="62" t="s">
-        <v>117</v>
-      </c>
-      <c r="B17" s="63">
-        <f>SUMPRODUCT(('📋 TODO'!A2:A55="BASE DE DONNÉES")*('📋 TODO'!E2:E55="Steeven")*('📋 TODO'!F2:F55))</f>
-        <v>45</v>
-      </c>
-      <c r="C17" s="64">
-        <f>SUMPRODUCT(('📋 TODO'!A2:A55="BASE DE DONNÉES")*('📋 TODO'!E2:E55="Mihaja")*('📋 TODO'!F2:F55))</f>
-        <v>60</v>
-      </c>
-      <c r="D17" s="65">
-        <f>SUMPRODUCT(('📋 TODO'!A2:A55="BASE DE DONNÉES")*('📋 TODO'!E2:E55="Aina")*('📋 TODO'!F2:F55))</f>
-        <v>0</v>
-      </c>
-      <c r="E17" s="66">
-        <f t="shared" si="1"/>
-        <v>105</v>
-      </c>
-    </row>
-    <row r="18" ht="19.5" customHeight="1">
-      <c r="A18" s="67" t="s">
-        <v>121</v>
-      </c>
-      <c r="B18" s="68">
-        <f>SUMPRODUCT(('📋 TODO'!A2:A55="NAVIGATION")*('📋 TODO'!E2:E55="Steeven")*('📋 TODO'!F2:F55))</f>
-        <v>0</v>
-      </c>
-      <c r="C18" s="69">
-        <f>SUMPRODUCT(('📋 TODO'!A2:A55="NAVIGATION")*('📋 TODO'!E2:E55="Mihaja")*('📋 TODO'!F2:F55))</f>
-        <v>0</v>
-      </c>
-      <c r="D18" s="70">
-        <f>SUMPRODUCT(('📋 TODO'!A2:A55="NAVIGATION")*('📋 TODO'!E2:E55="Aina")*('📋 TODO'!F2:F55))</f>
-        <v>120</v>
-      </c>
-      <c r="E18" s="27">
-        <f t="shared" si="1"/>
-        <v>120</v>
-      </c>
-    </row>
-    <row r="19" ht="19.5" customHeight="1">
-      <c r="A19" s="62" t="s">
-        <v>126</v>
-      </c>
-      <c r="B19" s="63">
-        <f>SUMPRODUCT(('📋 TODO'!A2:A55="TESTS &amp; LIVRAISON")*('📋 TODO'!E2:E55="Steeven")*('📋 TODO'!F2:F55))</f>
-        <v>60</v>
-      </c>
-      <c r="C19" s="64">
-        <f>SUMPRODUCT(('📋 TODO'!A2:A55="TESTS &amp; LIVRAISON")*('📋 TODO'!E2:E55="Mihaja")*('📋 TODO'!F2:F55))</f>
-        <v>60</v>
-      </c>
-      <c r="D19" s="65">
-        <f>SUMPRODUCT(('📋 TODO'!A2:A55="TESTS &amp; LIVRAISON")*('📋 TODO'!E2:E55="Aina")*('📋 TODO'!F2:F55))</f>
-        <v>45</v>
-      </c>
-      <c r="E19" s="66">
+      <c r="D19" s="43">
+        <f>SUMPRODUCT((' TODO'!A2:A53="TESTS &amp; LIVRAISON")*(' TODO'!E2:E53="Aina")*(' TODO'!F2:F53))</f>
+        <v>50</v>
+      </c>
+      <c r="E19" s="44">
         <f t="shared" si="1"/>
         <v>165</v>
       </c>
     </row>
     <row r="20" ht="21.75" customHeight="1">
       <c r="A20" s="37" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="B20" s="38">
         <f t="shared" ref="B20:E20" si="2">SUM(B3:B19)</f>
-        <v>1140</v>
+        <v>950</v>
       </c>
       <c r="C20" s="38">
         <f t="shared" si="2"/>
-        <v>870</v>
+        <v>845</v>
       </c>
       <c r="D20" s="38">
         <f t="shared" si="2"/>
-        <v>855</v>
+        <v>885</v>
       </c>
       <c r="E20" s="38">
         <f t="shared" si="2"/>
-        <v>2865</v>
+        <v>2680</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
     <row r="22" ht="25.5" customHeight="1">
       <c r="A22" s="28" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="B22" s="20"/>
       <c r="C22" s="20"/>
@@ -6140,77 +5576,77 @@
     </row>
     <row r="23" ht="27.75" customHeight="1">
       <c r="A23" s="22" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B23" s="22" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="C23" s="22" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="D23" s="22" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="E23" s="22" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
     </row>
     <row r="24" ht="19.5" customHeight="1">
       <c r="A24" s="23" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="B24" s="6">
-        <f>SUMPRODUCT(('📋 TODO'!E2:E55="Steeven")*('📋 TODO'!J2:J55="À FAIRE"))</f>
-        <v>25</v>
+        <f>SUMPRODUCT((' TODO'!E2:E53="Steeven")*(' TODO'!J2:J53="À FAIRE"))</f>
+        <v>20</v>
       </c>
       <c r="C24" s="6">
-        <f>SUMPRODUCT(('📋 TODO'!E2:E55="Steeven")*('📋 TODO'!J2:J55="EN COURS"))</f>
+        <f>SUMPRODUCT((' TODO'!E2:E53="Steeven")*(' TODO'!J2:J53="EN COURS"))</f>
         <v>0</v>
       </c>
       <c r="D24" s="6">
-        <f>SUMPRODUCT(('📋 TODO'!E2:E55="Steeven")*('📋 TODO'!J2:J55="OK"))</f>
+        <f>SUMPRODUCT((' TODO'!E2:E53="Steeven")*(' TODO'!J2:J53="OK"))</f>
         <v>0</v>
       </c>
       <c r="E24" s="8">
         <f t="shared" ref="E24:E26" si="3">SUM(B24:D24)</f>
-        <v>25</v>
+        <v>20</v>
       </c>
     </row>
     <row r="25" ht="19.5" customHeight="1">
-      <c r="A25" s="71" t="s">
-        <v>19</v>
+      <c r="A25" s="49" t="s">
+        <v>30</v>
       </c>
       <c r="B25" s="12">
-        <f>SUMPRODUCT(('📋 TODO'!E2:E55="Mihaja")*('📋 TODO'!J2:J55="À FAIRE"))</f>
-        <v>14</v>
+        <f>SUMPRODUCT((' TODO'!E2:E53="Mihaja")*(' TODO'!J2:J53="À FAIRE"))</f>
+        <v>17</v>
       </c>
       <c r="C25" s="12">
-        <f>SUMPRODUCT(('📋 TODO'!E2:E55="Mihaja")*('📋 TODO'!J2:J55="EN COURS"))</f>
+        <f>SUMPRODUCT((' TODO'!E2:E53="Mihaja")*(' TODO'!J2:J53="EN COURS"))</f>
         <v>0</v>
       </c>
       <c r="D25" s="12">
-        <f>SUMPRODUCT(('📋 TODO'!E2:E55="Mihaja")*('📋 TODO'!J2:J55="OK"))</f>
+        <f>SUMPRODUCT((' TODO'!E2:E53="Mihaja")*(' TODO'!J2:J53="OK"))</f>
         <v>0</v>
       </c>
       <c r="E25" s="14">
         <f t="shared" si="3"/>
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="26" ht="19.5" customHeight="1">
-      <c r="A26" s="72" t="s">
-        <v>14</v>
+      <c r="A26" s="50" t="s">
+        <v>35</v>
       </c>
       <c r="B26" s="6">
-        <f>SUMPRODUCT(('📋 TODO'!E2:E55="Aina")*('📋 TODO'!J2:J55="À FAIRE"))</f>
+        <f>SUMPRODUCT((' TODO'!E2:E53="Aina")*(' TODO'!J2:J53="À FAIRE"))</f>
         <v>15</v>
       </c>
       <c r="C26" s="6">
-        <f>SUMPRODUCT(('📋 TODO'!E2:E55="Aina")*('📋 TODO'!J2:J55="EN COURS"))</f>
+        <f>SUMPRODUCT((' TODO'!E2:E53="Aina")*(' TODO'!J2:J53="EN COURS"))</f>
         <v>0</v>
       </c>
       <c r="D26" s="6">
-        <f>SUMPRODUCT(('📋 TODO'!E2:E55="Aina")*('📋 TODO'!J2:J55="OK"))</f>
+        <f>SUMPRODUCT((' TODO'!E2:E53="Aina")*(' TODO'!J2:J53="OK"))</f>
         <v>0</v>
       </c>
       <c r="E26" s="8">
@@ -6220,11 +5656,11 @@
     </row>
     <row r="27" ht="21.75" customHeight="1">
       <c r="A27" s="37" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="B27" s="38">
         <f t="shared" ref="B27:E27" si="4">SUM(B24:B26)</f>
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C27" s="38">
         <f t="shared" si="4"/>
@@ -6236,7 +5672,7 @@
       </c>
       <c r="E27" s="38">
         <f t="shared" si="4"/>
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1"/>

</xml_diff>